<commit_message>
Embed BGP control-plane in 7 vEdge payloads and sync vEdge1-S400 live config; add EVE connection guide for AI, update timeline
</commit_message>
<xml_diff>
--- a/Template_Timeline_Tong_quan_08-08_den_21-11-2026.xlsx
+++ b/Template_Timeline_Tong_quan_08-08_den_21-11-2026.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -17,8 +17,11 @@
     <sheet name="Hướng dẫn sử dụng" sheetId="2" r:id="rId2"/>
     <sheet name="Gantt tuần" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -52,6 +55,9 @@
     <t>Sinh viên / Nhóm:</t>
   </si>
   <si>
+    <t>Trần Hữu Nhân - 52300235 , Nguyễn Nhật Hào - 523002198</t>
+  </si>
+  <si>
     <t>Giảng viên hướng dẫn:</t>
   </si>
   <si>
@@ -629,18 +635,14 @@
   </si>
   <si>
     <t>Nộp / trình bày</t>
-  </si>
-  <si>
-    <t>Trần Hữu Nhân - 52300235 , Nguyễn Nhật Hào - 523002198</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="165" formatCode="dd/mm"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -893,7 +895,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -904,7 +906,7 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -923,7 +925,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -969,10 +970,10 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
@@ -993,13 +994,13 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1008,7 +1009,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="12" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1017,7 +1018,7 @@
     <xf numFmtId="0" fontId="2" fillId="12" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="12" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="2" fillId="12" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="13" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1026,70 +1027,65 @@
     <xf numFmtId="0" fontId="2" fillId="13" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="13" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="2" fillId="13" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1102,9 +1098,16 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="3">
     <dxf>
@@ -1363,126 +1366,126 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15" customHeight="1">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
+      <c r="B1" s="70"/>
+      <c r="C1" s="70"/>
+      <c r="D1" s="70"/>
+      <c r="E1" s="70"/>
+      <c r="F1" s="70"/>
+      <c r="G1" s="70"/>
+      <c r="H1" s="70"/>
+      <c r="I1" s="70"/>
     </row>
     <row r="3" spans="1:9" ht="14.1" customHeight="1">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="58" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="54"/>
-      <c r="C3" s="53" t="s">
+      <c r="B3" s="71"/>
+      <c r="C3" s="65" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="54"/>
-      <c r="E3" s="54"/>
-      <c r="F3" s="54"/>
-      <c r="G3" s="63" t="s">
+      <c r="D3" s="71"/>
+      <c r="E3" s="71"/>
+      <c r="F3" s="71"/>
+      <c r="G3" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="54"/>
-      <c r="I3" s="37">
+      <c r="H3" s="71"/>
+      <c r="I3" s="36">
         <v>46242</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="14.1" customHeight="1">
-      <c r="A4" s="65" t="s">
+      <c r="A4" s="51" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="48"/>
-      <c r="C4" s="51" t="s">
-        <v>198</v>
-      </c>
-      <c r="D4" s="48"/>
-      <c r="E4" s="52" t="s">
+      <c r="B4" s="70"/>
+      <c r="C4" s="63" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="48"/>
-      <c r="G4" s="58" t="s">
+      <c r="D4" s="70"/>
+      <c r="E4" s="64" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="48"/>
-      <c r="I4" s="59"/>
+      <c r="F4" s="70"/>
+      <c r="G4" s="56" t="s">
+        <v>7</v>
+      </c>
+      <c r="H4" s="70"/>
+      <c r="I4" s="72"/>
     </row>
     <row r="5" spans="1:9" ht="14.1" customHeight="1">
-      <c r="A5" s="65" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="48"/>
-      <c r="C5" s="36">
+      <c r="A5" s="51" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="70"/>
+      <c r="C5" s="35">
         <v>46347</v>
       </c>
-      <c r="D5" s="66" t="s">
-        <v>8</v>
-      </c>
-      <c r="E5" s="48"/>
-      <c r="F5" s="35">
+      <c r="D5" s="54" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="70"/>
+      <c r="F5" s="34">
         <v>46332</v>
       </c>
-      <c r="G5" s="66" t="s">
-        <v>9</v>
-      </c>
-      <c r="H5" s="48"/>
-      <c r="I5" s="38" t="s">
+      <c r="G5" s="54" t="s">
         <v>10</v>
       </c>
+      <c r="H5" s="70"/>
+      <c r="I5" s="37" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="6" spans="1:9" ht="14.1" customHeight="1">
-      <c r="A6" s="49" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="50"/>
-      <c r="C6" s="60" t="s">
+      <c r="A6" s="62" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="50"/>
-      <c r="E6" s="50"/>
-      <c r="F6" s="50"/>
-      <c r="G6" s="50"/>
-      <c r="H6" s="50"/>
-      <c r="I6" s="61"/>
+      <c r="B6" s="73"/>
+      <c r="C6" s="57" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="73"/>
+      <c r="E6" s="73"/>
+      <c r="F6" s="73"/>
+      <c r="G6" s="73"/>
+      <c r="H6" s="73"/>
+      <c r="I6" s="74"/>
     </row>
     <row r="7" spans="1:9" ht="15" customHeight="1">
-      <c r="A7" s="47" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="48"/>
-      <c r="C7" s="48"/>
-      <c r="D7" s="48"/>
-      <c r="E7" s="48"/>
-      <c r="F7" s="48"/>
-      <c r="G7" s="48"/>
-      <c r="H7" s="48"/>
-      <c r="I7" s="48"/>
+      <c r="A7" s="61" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="70"/>
+      <c r="C7" s="70"/>
+      <c r="D7" s="70"/>
+      <c r="E7" s="70"/>
+      <c r="F7" s="70"/>
+      <c r="G7" s="70"/>
+      <c r="H7" s="70"/>
+      <c r="I7" s="70"/>
     </row>
     <row r="8" spans="1:9" ht="41.65" customHeight="1">
       <c r="A8" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F8" s="3"/>
       <c r="G8" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H8" s="3"/>
       <c r="I8" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="16.899999999999999" customHeight="1">
@@ -1490,772 +1493,787 @@
         <f>COUNTA(C13:C39)</f>
         <v>27</v>
       </c>
+      <c r="B9" s="46"/>
       <c r="C9" s="5">
         <f>COUNTIF(H13:H39,"Hoàn thành")</f>
         <v>7</v>
       </c>
+      <c r="D9" s="46"/>
       <c r="E9" s="5">
         <f>COUNTIF(H13:H39,"Đang thực hiện")</f>
         <v>3</v>
       </c>
+      <c r="F9" s="46"/>
       <c r="G9" s="5">
         <f>COUNTIF(H13:H39,"Chưa bắt đầu")</f>
         <v>17</v>
       </c>
+      <c r="H9" s="46"/>
       <c r="I9" s="4">
         <v>46332</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="19.149999999999999" customHeight="1">
       <c r="A11" s="7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I11" s="9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:9">
       <c r="A12" s="10"/>
-      <c r="I12" s="11"/>
+      <c r="B12" s="46"/>
+      <c r="C12" s="46"/>
+      <c r="D12" s="46"/>
+      <c r="E12" s="46"/>
+      <c r="F12" s="46"/>
+      <c r="G12" s="46"/>
+      <c r="H12" s="46"/>
+      <c r="I12" s="47"/>
     </row>
     <row r="13" spans="1:9" ht="40.5" customHeight="1">
-      <c r="A13" s="14">
+      <c r="A13" s="13">
         <v>1</v>
       </c>
-      <c r="B13" s="64" t="s">
-        <v>28</v>
-      </c>
-      <c r="C13" s="39" t="s">
+      <c r="B13" s="60" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="39" t="s">
+      <c r="C13" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="E13" s="40">
+      <c r="D13" s="38" t="s">
+        <v>31</v>
+      </c>
+      <c r="E13" s="39">
         <v>46242</v>
       </c>
-      <c r="F13" s="40">
+      <c r="F13" s="39">
         <v>46242</v>
       </c>
-      <c r="G13" s="39" t="s">
-        <v>31</v>
-      </c>
-      <c r="H13" s="39" t="s">
+      <c r="G13" s="38" t="s">
+        <v>32</v>
+      </c>
+      <c r="H13" s="38" t="s">
+        <v>16</v>
+      </c>
+      <c r="I13" s="38" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="40.5" customHeight="1">
+      <c r="A14" s="13">
+        <v>2</v>
+      </c>
+      <c r="B14" s="75"/>
+      <c r="C14" s="38" t="s">
+        <v>34</v>
+      </c>
+      <c r="D14" s="38" t="s">
+        <v>35</v>
+      </c>
+      <c r="E14" s="39">
+        <v>46242</v>
+      </c>
+      <c r="F14" s="39">
+        <v>46246</v>
+      </c>
+      <c r="G14" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="H14" s="38" t="s">
+        <v>16</v>
+      </c>
+      <c r="I14" s="38" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="40.5" customHeight="1">
+      <c r="A15" s="13">
+        <v>3</v>
+      </c>
+      <c r="B15" s="75"/>
+      <c r="C15" s="38" t="s">
+        <v>38</v>
+      </c>
+      <c r="D15" s="38" t="s">
+        <v>39</v>
+      </c>
+      <c r="E15" s="39">
+        <v>46242</v>
+      </c>
+      <c r="F15" s="39">
+        <v>46246</v>
+      </c>
+      <c r="G15" s="38" t="s">
+        <v>40</v>
+      </c>
+      <c r="H15" s="38" t="s">
+        <v>16</v>
+      </c>
+      <c r="I15" s="38" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="40.5" customHeight="1">
+      <c r="A16" s="13">
+        <v>4</v>
+      </c>
+      <c r="B16" s="76"/>
+      <c r="C16" s="38" t="s">
+        <v>42</v>
+      </c>
+      <c r="D16" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="E16" s="39">
+        <v>46242</v>
+      </c>
+      <c r="F16" s="39">
+        <v>46246</v>
+      </c>
+      <c r="G16" s="38" t="s">
+        <v>44</v>
+      </c>
+      <c r="H16" s="38" t="s">
+        <v>16</v>
+      </c>
+      <c r="I16" s="38" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="40.5" customHeight="1">
+      <c r="A17" s="13">
+        <v>5</v>
+      </c>
+      <c r="B17" s="55" t="s">
+        <v>46</v>
+      </c>
+      <c r="C17" s="38" t="s">
+        <v>47</v>
+      </c>
+      <c r="D17" s="38" t="s">
+        <v>48</v>
+      </c>
+      <c r="E17" s="39">
+        <v>46242</v>
+      </c>
+      <c r="F17" s="39">
+        <v>46246</v>
+      </c>
+      <c r="G17" s="38" t="s">
+        <v>49</v>
+      </c>
+      <c r="H17" s="38" t="s">
+        <v>16</v>
+      </c>
+      <c r="I17" s="38" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="40.5" customHeight="1">
+      <c r="A18" s="13">
+        <v>6</v>
+      </c>
+      <c r="B18" s="75"/>
+      <c r="C18" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="D18" s="38" t="s">
+        <v>52</v>
+      </c>
+      <c r="E18" s="39">
+        <v>46242</v>
+      </c>
+      <c r="F18" s="39">
+        <v>46246</v>
+      </c>
+      <c r="G18" s="38" t="s">
+        <v>53</v>
+      </c>
+      <c r="H18" s="38" t="s">
+        <v>16</v>
+      </c>
+      <c r="I18" s="38" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="27" customHeight="1">
+      <c r="A19" s="13">
+        <v>7</v>
+      </c>
+      <c r="B19" s="75"/>
+      <c r="C19" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="D19" s="38" t="s">
+        <v>56</v>
+      </c>
+      <c r="E19" s="39">
+        <v>46261</v>
+      </c>
+      <c r="F19" s="39">
+        <v>46270</v>
+      </c>
+      <c r="G19" s="38" t="s">
+        <v>57</v>
+      </c>
+      <c r="H19" s="38" t="s">
+        <v>18</v>
+      </c>
+      <c r="I19" s="38"/>
+    </row>
+    <row r="20" spans="1:9" ht="40.5" customHeight="1">
+      <c r="A20" s="13">
+        <v>8</v>
+      </c>
+      <c r="B20" s="76"/>
+      <c r="C20" s="38" t="s">
+        <v>58</v>
+      </c>
+      <c r="D20" s="38" t="s">
+        <v>59</v>
+      </c>
+      <c r="E20" s="39">
+        <v>46242</v>
+      </c>
+      <c r="F20" s="39">
+        <v>46246</v>
+      </c>
+      <c r="G20" s="38" t="s">
+        <v>60</v>
+      </c>
+      <c r="H20" s="38" t="s">
+        <v>16</v>
+      </c>
+      <c r="I20" s="38" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="27.75" customHeight="1">
+      <c r="A21" s="13">
+        <v>9</v>
+      </c>
+      <c r="B21" s="52" t="s">
+        <v>62</v>
+      </c>
+      <c r="C21" s="38" t="s">
+        <v>63</v>
+      </c>
+      <c r="D21" s="38" t="s">
+        <v>64</v>
+      </c>
+      <c r="E21" s="39">
+        <v>46242</v>
+      </c>
+      <c r="F21" s="39">
+        <v>46277</v>
+      </c>
+      <c r="G21" s="38" t="s">
+        <v>65</v>
+      </c>
+      <c r="H21" s="38" t="s">
+        <v>17</v>
+      </c>
+      <c r="I21" s="38" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="40.5" customHeight="1">
+      <c r="A22" s="13">
+        <v>10</v>
+      </c>
+      <c r="B22" s="75"/>
+      <c r="C22" s="38" t="s">
+        <v>67</v>
+      </c>
+      <c r="D22" s="38" t="s">
+        <v>68</v>
+      </c>
+      <c r="E22" s="39">
+        <v>46242</v>
+      </c>
+      <c r="F22" s="39">
+        <v>46284</v>
+      </c>
+      <c r="G22" s="38" t="s">
+        <v>69</v>
+      </c>
+      <c r="H22" s="38" t="s">
+        <v>17</v>
+      </c>
+      <c r="I22" s="38" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="27.75" customHeight="1">
+      <c r="A23" s="13">
+        <v>11</v>
+      </c>
+      <c r="B23" s="75"/>
+      <c r="C23" s="38" t="s">
+        <v>71</v>
+      </c>
+      <c r="D23" s="38" t="s">
+        <v>72</v>
+      </c>
+      <c r="E23" s="39">
+        <v>46285</v>
+      </c>
+      <c r="F23" s="39">
+        <v>46291</v>
+      </c>
+      <c r="G23" s="38" t="s">
+        <v>73</v>
+      </c>
+      <c r="H23" s="38" t="s">
+        <v>18</v>
+      </c>
+      <c r="I23" s="38"/>
+    </row>
+    <row r="24" spans="1:9" ht="40.5" customHeight="1">
+      <c r="A24" s="13">
+        <v>12</v>
+      </c>
+      <c r="B24" s="75"/>
+      <c r="C24" s="38" t="s">
+        <v>74</v>
+      </c>
+      <c r="D24" s="38" t="s">
+        <v>75</v>
+      </c>
+      <c r="E24" s="39">
+        <v>46292</v>
+      </c>
+      <c r="F24" s="39">
+        <v>46298</v>
+      </c>
+      <c r="G24" s="38" t="s">
+        <v>76</v>
+      </c>
+      <c r="H24" s="38" t="s">
+        <v>18</v>
+      </c>
+      <c r="I24" s="38"/>
+    </row>
+    <row r="25" spans="1:9" ht="40.5" customHeight="1">
+      <c r="A25" s="13">
+        <v>13</v>
+      </c>
+      <c r="B25" s="76"/>
+      <c r="C25" s="38" t="s">
+        <v>77</v>
+      </c>
+      <c r="D25" s="38" t="s">
+        <v>78</v>
+      </c>
+      <c r="E25" s="39">
+        <v>46242</v>
+      </c>
+      <c r="F25" s="39">
+        <v>46298</v>
+      </c>
+      <c r="G25" s="38" t="s">
+        <v>79</v>
+      </c>
+      <c r="H25" s="38" t="s">
+        <v>17</v>
+      </c>
+      <c r="I25" s="38" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="27" customHeight="1">
+      <c r="A26" s="13">
+        <v>14</v>
+      </c>
+      <c r="B26" s="53" t="s">
+        <v>81</v>
+      </c>
+      <c r="C26" s="38" t="s">
+        <v>82</v>
+      </c>
+      <c r="D26" s="38" t="s">
+        <v>83</v>
+      </c>
+      <c r="E26" s="39">
+        <v>46299</v>
+      </c>
+      <c r="F26" s="39">
+        <v>46305</v>
+      </c>
+      <c r="G26" s="38" t="s">
+        <v>84</v>
+      </c>
+      <c r="H26" s="38" t="s">
+        <v>18</v>
+      </c>
+      <c r="I26" s="38"/>
+    </row>
+    <row r="27" spans="1:9" ht="40.5" customHeight="1">
+      <c r="A27" s="13">
         <v>15</v>
       </c>
-      <c r="I13" s="39" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="40.5" customHeight="1">
-      <c r="A14" s="14">
-        <v>2</v>
-      </c>
-      <c r="B14" s="56"/>
-      <c r="C14" s="39" t="s">
-        <v>33</v>
-      </c>
-      <c r="D14" s="39" t="s">
-        <v>34</v>
-      </c>
-      <c r="E14" s="40">
-        <v>46242</v>
-      </c>
-      <c r="F14" s="40">
-        <v>46246</v>
-      </c>
-      <c r="G14" s="39" t="s">
-        <v>35</v>
-      </c>
-      <c r="H14" s="39" t="s">
-        <v>15</v>
-      </c>
-      <c r="I14" s="39" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="40.5" customHeight="1">
-      <c r="A15" s="14">
-        <v>3</v>
-      </c>
-      <c r="B15" s="56"/>
-      <c r="C15" s="39" t="s">
-        <v>37</v>
-      </c>
-      <c r="D15" s="39" t="s">
-        <v>38</v>
-      </c>
-      <c r="E15" s="40">
-        <v>46242</v>
-      </c>
-      <c r="F15" s="40">
-        <v>46246</v>
-      </c>
-      <c r="G15" s="39" t="s">
-        <v>39</v>
-      </c>
-      <c r="H15" s="39" t="s">
-        <v>15</v>
-      </c>
-      <c r="I15" s="39" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="40.5" customHeight="1">
-      <c r="A16" s="14">
-        <v>4</v>
-      </c>
-      <c r="B16" s="57"/>
-      <c r="C16" s="39" t="s">
-        <v>41</v>
-      </c>
-      <c r="D16" s="39" t="s">
-        <v>42</v>
-      </c>
-      <c r="E16" s="40">
-        <v>46242</v>
-      </c>
-      <c r="F16" s="40">
-        <v>46246</v>
-      </c>
-      <c r="G16" s="39" t="s">
-        <v>43</v>
-      </c>
-      <c r="H16" s="39" t="s">
-        <v>15</v>
-      </c>
-      <c r="I16" s="39" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" ht="40.5" customHeight="1">
-      <c r="A17" s="14">
-        <v>5</v>
-      </c>
-      <c r="B17" s="55" t="s">
-        <v>45</v>
-      </c>
-      <c r="C17" s="39" t="s">
-        <v>46</v>
-      </c>
-      <c r="D17" s="39" t="s">
-        <v>47</v>
-      </c>
-      <c r="E17" s="40">
-        <v>46242</v>
-      </c>
-      <c r="F17" s="40">
-        <v>46246</v>
-      </c>
-      <c r="G17" s="39" t="s">
-        <v>48</v>
-      </c>
-      <c r="H17" s="39" t="s">
-        <v>15</v>
-      </c>
-      <c r="I17" s="39" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" ht="40.5" customHeight="1">
-      <c r="A18" s="14">
-        <v>6</v>
-      </c>
-      <c r="B18" s="56"/>
-      <c r="C18" s="39" t="s">
-        <v>50</v>
-      </c>
-      <c r="D18" s="39" t="s">
-        <v>51</v>
-      </c>
-      <c r="E18" s="40">
-        <v>46242</v>
-      </c>
-      <c r="F18" s="40">
-        <v>46246</v>
-      </c>
-      <c r="G18" s="39" t="s">
-        <v>52</v>
-      </c>
-      <c r="H18" s="39" t="s">
-        <v>15</v>
-      </c>
-      <c r="I18" s="39" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" ht="27" customHeight="1">
-      <c r="A19" s="14">
-        <v>7</v>
-      </c>
-      <c r="B19" s="56"/>
-      <c r="C19" s="39" t="s">
-        <v>54</v>
-      </c>
-      <c r="D19" s="39" t="s">
-        <v>55</v>
-      </c>
-      <c r="E19" s="40">
-        <v>46261</v>
-      </c>
-      <c r="F19" s="40">
-        <v>46270</v>
-      </c>
-      <c r="G19" s="39" t="s">
-        <v>56</v>
-      </c>
-      <c r="H19" s="39" t="s">
+      <c r="B27" s="75"/>
+      <c r="C27" s="38" t="s">
+        <v>85</v>
+      </c>
+      <c r="D27" s="38" t="s">
+        <v>86</v>
+      </c>
+      <c r="E27" s="39">
+        <v>46306</v>
+      </c>
+      <c r="F27" s="39">
+        <v>46312</v>
+      </c>
+      <c r="G27" s="38" t="s">
+        <v>87</v>
+      </c>
+      <c r="H27" s="38" t="s">
+        <v>18</v>
+      </c>
+      <c r="I27" s="38"/>
+    </row>
+    <row r="28" spans="1:9" ht="40.5" customHeight="1">
+      <c r="A28" s="13">
+        <v>16</v>
+      </c>
+      <c r="B28" s="75"/>
+      <c r="C28" s="38" t="s">
+        <v>88</v>
+      </c>
+      <c r="D28" s="38" t="s">
+        <v>89</v>
+      </c>
+      <c r="E28" s="39">
+        <v>46313</v>
+      </c>
+      <c r="F28" s="39">
+        <v>46319</v>
+      </c>
+      <c r="G28" s="38" t="s">
+        <v>90</v>
+      </c>
+      <c r="H28" s="38" t="s">
+        <v>18</v>
+      </c>
+      <c r="I28" s="38"/>
+    </row>
+    <row r="29" spans="1:9" ht="27" customHeight="1">
+      <c r="A29" s="13">
         <v>17</v>
       </c>
-      <c r="I19" s="39"/>
-    </row>
-    <row r="20" spans="1:9" ht="40.5" customHeight="1">
-      <c r="A20" s="14">
-        <v>8</v>
-      </c>
-      <c r="B20" s="57"/>
-      <c r="C20" s="39" t="s">
-        <v>57</v>
-      </c>
-      <c r="D20" s="39" t="s">
-        <v>58</v>
-      </c>
-      <c r="E20" s="40">
-        <v>46242</v>
-      </c>
-      <c r="F20" s="40">
-        <v>46246</v>
-      </c>
-      <c r="G20" s="39" t="s">
-        <v>59</v>
-      </c>
-      <c r="H20" s="39" t="s">
-        <v>15</v>
-      </c>
-      <c r="I20" s="39" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" ht="27.75" customHeight="1">
-      <c r="A21" s="14">
-        <v>9</v>
-      </c>
-      <c r="B21" s="68" t="s">
-        <v>61</v>
-      </c>
-      <c r="C21" s="39" t="s">
-        <v>62</v>
-      </c>
-      <c r="D21" s="39" t="s">
-        <v>63</v>
-      </c>
-      <c r="E21" s="40">
-        <v>46242</v>
-      </c>
-      <c r="F21" s="40">
-        <v>46277</v>
-      </c>
-      <c r="G21" s="39" t="s">
-        <v>64</v>
-      </c>
-      <c r="H21" s="39" t="s">
-        <v>16</v>
-      </c>
-      <c r="I21" s="39" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" ht="40.5" customHeight="1">
-      <c r="A22" s="14">
-        <v>10</v>
-      </c>
-      <c r="B22" s="56"/>
-      <c r="C22" s="39" t="s">
-        <v>66</v>
-      </c>
-      <c r="D22" s="39" t="s">
-        <v>67</v>
-      </c>
-      <c r="E22" s="40">
-        <v>46242</v>
-      </c>
-      <c r="F22" s="40">
-        <v>46284</v>
-      </c>
-      <c r="G22" s="39" t="s">
-        <v>68</v>
-      </c>
-      <c r="H22" s="39" t="s">
-        <v>16</v>
-      </c>
-      <c r="I22" s="39" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" ht="27.75" customHeight="1">
-      <c r="A23" s="14">
-        <v>11</v>
-      </c>
-      <c r="B23" s="56"/>
-      <c r="C23" s="39" t="s">
-        <v>70</v>
-      </c>
-      <c r="D23" s="39" t="s">
-        <v>71</v>
-      </c>
-      <c r="E23" s="40">
-        <v>46285</v>
-      </c>
-      <c r="F23" s="40">
-        <v>46291</v>
-      </c>
-      <c r="G23" s="39" t="s">
-        <v>72</v>
-      </c>
-      <c r="H23" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="I23" s="39"/>
-    </row>
-    <row r="24" spans="1:9" ht="40.5" customHeight="1">
-      <c r="A24" s="14">
-        <v>12</v>
-      </c>
-      <c r="B24" s="56"/>
-      <c r="C24" s="39" t="s">
-        <v>73</v>
-      </c>
-      <c r="D24" s="39" t="s">
-        <v>74</v>
-      </c>
-      <c r="E24" s="40">
-        <v>46292</v>
-      </c>
-      <c r="F24" s="40">
-        <v>46298</v>
-      </c>
-      <c r="G24" s="39" t="s">
-        <v>75</v>
-      </c>
-      <c r="H24" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="I24" s="39"/>
-    </row>
-    <row r="25" spans="1:9" ht="40.5" customHeight="1">
-      <c r="A25" s="14">
-        <v>13</v>
-      </c>
-      <c r="B25" s="57"/>
-      <c r="C25" s="39" t="s">
-        <v>76</v>
-      </c>
-      <c r="D25" s="39" t="s">
-        <v>77</v>
-      </c>
-      <c r="E25" s="40">
-        <v>46242</v>
-      </c>
-      <c r="F25" s="40">
-        <v>46298</v>
-      </c>
-      <c r="G25" s="39" t="s">
-        <v>78</v>
-      </c>
-      <c r="H25" s="39" t="s">
-        <v>16</v>
-      </c>
-      <c r="I25" s="39" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" ht="27" customHeight="1">
-      <c r="A26" s="14">
-        <v>14</v>
-      </c>
-      <c r="B26" s="69" t="s">
-        <v>80</v>
-      </c>
-      <c r="C26" s="39" t="s">
-        <v>81</v>
-      </c>
-      <c r="D26" s="39" t="s">
-        <v>82</v>
-      </c>
-      <c r="E26" s="40">
+      <c r="B29" s="76"/>
+      <c r="C29" s="38" t="s">
+        <v>91</v>
+      </c>
+      <c r="D29" s="38" t="s">
+        <v>92</v>
+      </c>
+      <c r="E29" s="39">
+        <v>46317</v>
+      </c>
+      <c r="F29" s="39">
+        <v>46323</v>
+      </c>
+      <c r="G29" s="38" t="s">
+        <v>93</v>
+      </c>
+      <c r="H29" s="38" t="s">
+        <v>18</v>
+      </c>
+      <c r="I29" s="38"/>
+    </row>
+    <row r="30" spans="1:9" ht="40.5" customHeight="1">
+      <c r="A30" s="13">
+        <v>18</v>
+      </c>
+      <c r="B30" s="50" t="s">
+        <v>94</v>
+      </c>
+      <c r="C30" s="38" t="s">
+        <v>95</v>
+      </c>
+      <c r="D30" s="38" t="s">
+        <v>96</v>
+      </c>
+      <c r="E30" s="39">
         <v>46299</v>
       </c>
-      <c r="F26" s="40">
-        <v>46305</v>
-      </c>
-      <c r="G26" s="39" t="s">
-        <v>83</v>
-      </c>
-      <c r="H26" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="I26" s="39"/>
-    </row>
-    <row r="27" spans="1:9" ht="40.5" customHeight="1">
-      <c r="A27" s="14">
-        <v>15</v>
-      </c>
-      <c r="B27" s="56"/>
-      <c r="C27" s="39" t="s">
-        <v>84</v>
-      </c>
-      <c r="D27" s="39" t="s">
-        <v>85</v>
-      </c>
-      <c r="E27" s="40">
-        <v>46306</v>
-      </c>
-      <c r="F27" s="40">
+      <c r="F30" s="39">
         <v>46312</v>
       </c>
-      <c r="G27" s="39" t="s">
-        <v>86</v>
-      </c>
-      <c r="H27" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="I27" s="39"/>
-    </row>
-    <row r="28" spans="1:9" ht="40.5" customHeight="1">
-      <c r="A28" s="14">
-        <v>16</v>
-      </c>
-      <c r="B28" s="56"/>
-      <c r="C28" s="39" t="s">
-        <v>87</v>
-      </c>
-      <c r="D28" s="39" t="s">
-        <v>88</v>
-      </c>
-      <c r="E28" s="40">
+      <c r="G30" s="38" t="s">
+        <v>97</v>
+      </c>
+      <c r="H30" s="38" t="s">
+        <v>18</v>
+      </c>
+      <c r="I30" s="38"/>
+    </row>
+    <row r="31" spans="1:9" ht="27.75" customHeight="1">
+      <c r="A31" s="13">
+        <v>19</v>
+      </c>
+      <c r="B31" s="75"/>
+      <c r="C31" s="38" t="s">
+        <v>98</v>
+      </c>
+      <c r="D31" s="38" t="s">
+        <v>99</v>
+      </c>
+      <c r="E31" s="39">
         <v>46313</v>
       </c>
-      <c r="F28" s="40">
-        <v>46319</v>
-      </c>
-      <c r="G28" s="39" t="s">
-        <v>89</v>
-      </c>
-      <c r="H28" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="I28" s="39"/>
-    </row>
-    <row r="29" spans="1:9" ht="27" customHeight="1">
-      <c r="A29" s="14">
-        <v>17</v>
-      </c>
-      <c r="B29" s="57"/>
-      <c r="C29" s="39" t="s">
-        <v>90</v>
-      </c>
-      <c r="D29" s="39" t="s">
-        <v>91</v>
-      </c>
-      <c r="E29" s="40">
-        <v>46317</v>
-      </c>
-      <c r="F29" s="40">
+      <c r="F31" s="39">
         <v>46323</v>
       </c>
-      <c r="G29" s="39" t="s">
-        <v>92</v>
-      </c>
-      <c r="H29" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="I29" s="39"/>
-    </row>
-    <row r="30" spans="1:9" ht="40.5" customHeight="1">
-      <c r="A30" s="14">
+      <c r="G31" s="38" t="s">
+        <v>100</v>
+      </c>
+      <c r="H31" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="B30" s="67" t="s">
-        <v>93</v>
-      </c>
-      <c r="C30" s="39" t="s">
+      <c r="I31" s="38"/>
+    </row>
+    <row r="32" spans="1:9" ht="27.75" customHeight="1">
+      <c r="A32" s="13">
+        <v>20</v>
+      </c>
+      <c r="B32" s="75"/>
+      <c r="C32" s="38" t="s">
+        <v>101</v>
+      </c>
+      <c r="D32" s="38" t="s">
+        <v>102</v>
+      </c>
+      <c r="E32" s="39">
+        <v>46324</v>
+      </c>
+      <c r="F32" s="39">
+        <v>46326</v>
+      </c>
+      <c r="G32" s="38" t="s">
+        <v>103</v>
+      </c>
+      <c r="H32" s="38" t="s">
+        <v>18</v>
+      </c>
+      <c r="I32" s="38"/>
+    </row>
+    <row r="33" spans="1:9" ht="40.5" customHeight="1">
+      <c r="A33" s="13">
+        <v>21</v>
+      </c>
+      <c r="B33" s="76"/>
+      <c r="C33" s="38" t="s">
+        <v>104</v>
+      </c>
+      <c r="D33" s="38" t="s">
+        <v>105</v>
+      </c>
+      <c r="E33" s="39">
+        <v>46327</v>
+      </c>
+      <c r="F33" s="39">
+        <v>46330</v>
+      </c>
+      <c r="G33" s="38" t="s">
+        <v>106</v>
+      </c>
+      <c r="H33" s="38" t="s">
+        <v>18</v>
+      </c>
+      <c r="I33" s="38"/>
+    </row>
+    <row r="34" spans="1:9" ht="55.5" customHeight="1">
+      <c r="A34" s="14">
+        <v>22</v>
+      </c>
+      <c r="B34" s="40" t="s">
         <v>94</v>
       </c>
-      <c r="D30" s="39" t="s">
-        <v>95</v>
-      </c>
-      <c r="E30" s="40">
-        <v>46299</v>
-      </c>
-      <c r="F30" s="40">
-        <v>46312</v>
-      </c>
-      <c r="G30" s="39" t="s">
-        <v>96</v>
-      </c>
-      <c r="H30" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="I30" s="39"/>
-    </row>
-    <row r="31" spans="1:9" ht="27.75" customHeight="1">
-      <c r="A31" s="14">
-        <v>19</v>
-      </c>
-      <c r="B31" s="56"/>
-      <c r="C31" s="39" t="s">
-        <v>97</v>
-      </c>
-      <c r="D31" s="39" t="s">
-        <v>98</v>
-      </c>
-      <c r="E31" s="40">
-        <v>46313</v>
-      </c>
-      <c r="F31" s="40">
-        <v>46323</v>
-      </c>
-      <c r="G31" s="39" t="s">
-        <v>99</v>
-      </c>
-      <c r="H31" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="I31" s="39"/>
-    </row>
-    <row r="32" spans="1:9" ht="27.75" customHeight="1">
-      <c r="A32" s="14">
-        <v>20</v>
-      </c>
-      <c r="B32" s="56"/>
-      <c r="C32" s="39" t="s">
-        <v>100</v>
-      </c>
-      <c r="D32" s="39" t="s">
-        <v>101</v>
-      </c>
-      <c r="E32" s="40">
-        <v>46324</v>
-      </c>
-      <c r="F32" s="40">
-        <v>46326</v>
-      </c>
-      <c r="G32" s="39" t="s">
-        <v>102</v>
-      </c>
-      <c r="H32" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="I32" s="39"/>
-    </row>
-    <row r="33" spans="1:9" ht="40.5" customHeight="1">
-      <c r="A33" s="14">
-        <v>21</v>
-      </c>
-      <c r="B33" s="57"/>
-      <c r="C33" s="39" t="s">
-        <v>103</v>
-      </c>
-      <c r="D33" s="39" t="s">
-        <v>104</v>
-      </c>
-      <c r="E33" s="40">
-        <v>46327</v>
-      </c>
-      <c r="F33" s="40">
-        <v>46330</v>
-      </c>
-      <c r="G33" s="39" t="s">
-        <v>105</v>
-      </c>
-      <c r="H33" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="I33" s="39"/>
-    </row>
-    <row r="34" spans="1:9" ht="55.5" customHeight="1">
-      <c r="A34" s="15">
-        <v>22</v>
-      </c>
-      <c r="B34" s="41" t="s">
-        <v>93</v>
-      </c>
-      <c r="C34" s="42" t="s">
-        <v>106</v>
-      </c>
-      <c r="D34" s="42" t="s">
+      <c r="C34" s="41" t="s">
         <v>107</v>
       </c>
-      <c r="E34" s="43">
+      <c r="D34" s="41" t="s">
+        <v>108</v>
+      </c>
+      <c r="E34" s="42">
         <v>46331</v>
       </c>
-      <c r="F34" s="43">
+      <c r="F34" s="42">
         <v>46332</v>
       </c>
-      <c r="G34" s="42" t="s">
-        <v>108</v>
-      </c>
-      <c r="H34" s="42" t="s">
-        <v>17</v>
-      </c>
-      <c r="I34" s="42" t="s">
+      <c r="G34" s="41" t="s">
         <v>109</v>
       </c>
+      <c r="H34" s="41" t="s">
+        <v>18</v>
+      </c>
+      <c r="I34" s="41" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="35" spans="1:9" ht="40.5" customHeight="1">
-      <c r="A35" s="14">
+      <c r="A35" s="13">
         <v>23</v>
       </c>
-      <c r="B35" s="71" t="s">
-        <v>110</v>
-      </c>
-      <c r="C35" s="39" t="s">
+      <c r="B35" s="49" t="s">
         <v>111</v>
       </c>
-      <c r="D35" s="39" t="s">
+      <c r="C35" s="38" t="s">
         <v>112</v>
       </c>
-      <c r="E35" s="40">
+      <c r="D35" s="38" t="s">
+        <v>113</v>
+      </c>
+      <c r="E35" s="39">
         <v>46333</v>
       </c>
-      <c r="F35" s="40">
+      <c r="F35" s="39">
         <v>46339</v>
       </c>
-      <c r="G35" s="39" t="s">
-        <v>113</v>
-      </c>
-      <c r="H35" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="I35" s="39"/>
+      <c r="G35" s="38" t="s">
+        <v>114</v>
+      </c>
+      <c r="H35" s="38" t="s">
+        <v>18</v>
+      </c>
+      <c r="I35" s="38"/>
     </row>
     <row r="36" spans="1:9" ht="27.75" customHeight="1">
-      <c r="A36" s="14">
+      <c r="A36" s="13">
         <v>24</v>
       </c>
-      <c r="B36" s="56"/>
-      <c r="C36" s="39" t="s">
-        <v>114</v>
-      </c>
-      <c r="D36" s="39" t="s">
+      <c r="B36" s="75"/>
+      <c r="C36" s="38" t="s">
         <v>115</v>
       </c>
-      <c r="E36" s="40">
+      <c r="D36" s="38" t="s">
+        <v>116</v>
+      </c>
+      <c r="E36" s="39">
         <v>46333</v>
       </c>
-      <c r="F36" s="40">
+      <c r="F36" s="39">
         <v>46340</v>
       </c>
-      <c r="G36" s="39" t="s">
-        <v>116</v>
-      </c>
-      <c r="H36" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="I36" s="39"/>
+      <c r="G36" s="38" t="s">
+        <v>117</v>
+      </c>
+      <c r="H36" s="38" t="s">
+        <v>18</v>
+      </c>
+      <c r="I36" s="38"/>
     </row>
     <row r="37" spans="1:9" ht="40.5" customHeight="1">
-      <c r="A37" s="14">
+      <c r="A37" s="13">
         <v>25</v>
       </c>
-      <c r="B37" s="56"/>
-      <c r="C37" s="39" t="s">
-        <v>117</v>
-      </c>
-      <c r="D37" s="39" t="s">
+      <c r="B37" s="75"/>
+      <c r="C37" s="38" t="s">
         <v>118</v>
       </c>
-      <c r="E37" s="40">
+      <c r="D37" s="38" t="s">
+        <v>119</v>
+      </c>
+      <c r="E37" s="39">
         <v>46340</v>
       </c>
-      <c r="F37" s="40">
+      <c r="F37" s="39">
         <v>46343</v>
       </c>
-      <c r="G37" s="39" t="s">
-        <v>119</v>
-      </c>
-      <c r="H37" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="I37" s="39"/>
+      <c r="G37" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="H37" s="38" t="s">
+        <v>18</v>
+      </c>
+      <c r="I37" s="38"/>
     </row>
     <row r="38" spans="1:9" ht="40.5" customHeight="1">
-      <c r="A38" s="14">
+      <c r="A38" s="13">
         <v>26</v>
       </c>
-      <c r="B38" s="57"/>
-      <c r="C38" s="39" t="s">
-        <v>120</v>
-      </c>
-      <c r="D38" s="39" t="s">
+      <c r="B38" s="76"/>
+      <c r="C38" s="38" t="s">
         <v>121</v>
       </c>
-      <c r="E38" s="40">
+      <c r="D38" s="38" t="s">
+        <v>122</v>
+      </c>
+      <c r="E38" s="39">
         <v>46344</v>
       </c>
-      <c r="F38" s="40">
+      <c r="F38" s="39">
         <v>46346</v>
       </c>
-      <c r="G38" s="39" t="s">
-        <v>122</v>
-      </c>
-      <c r="H38" s="39" t="s">
-        <v>17</v>
-      </c>
-      <c r="I38" s="39"/>
+      <c r="G38" s="38" t="s">
+        <v>123</v>
+      </c>
+      <c r="H38" s="38" t="s">
+        <v>18</v>
+      </c>
+      <c r="I38" s="38"/>
     </row>
     <row r="39" spans="1:9" ht="27.75" customHeight="1">
-      <c r="A39" s="16">
+      <c r="A39" s="15">
         <v>27</v>
       </c>
-      <c r="B39" s="44" t="s">
-        <v>110</v>
-      </c>
-      <c r="C39" s="45" t="s">
-        <v>123</v>
-      </c>
-      <c r="D39" s="45" t="s">
+      <c r="B39" s="43" t="s">
+        <v>111</v>
+      </c>
+      <c r="C39" s="44" t="s">
         <v>124</v>
       </c>
-      <c r="E39" s="46">
+      <c r="D39" s="44" t="s">
+        <v>125</v>
+      </c>
+      <c r="E39" s="45">
         <v>46347</v>
       </c>
-      <c r="F39" s="46">
+      <c r="F39" s="45">
         <v>46347</v>
       </c>
-      <c r="G39" s="45" t="s">
-        <v>125</v>
-      </c>
-      <c r="H39" s="45" t="s">
-        <v>17</v>
-      </c>
-      <c r="I39" s="45" t="s">
+      <c r="G39" s="44" t="s">
         <v>126</v>
+      </c>
+      <c r="H39" s="44" t="s">
+        <v>18</v>
+      </c>
+      <c r="I39" s="44" t="s">
+        <v>127</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="C3:F3"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="B35:B38"/>
     <mergeCell ref="B30:B33"/>
@@ -2272,10 +2290,6 @@
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="G5:H5"/>
     <mergeCell ref="A7:I7"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="C3:F3"/>
   </mergeCells>
   <conditionalFormatting sqref="H13:H39">
     <cfRule type="expression" dxfId="2" priority="1">
@@ -2310,236 +2324,236 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="20.65" customHeight="1">
-      <c r="A1" s="73" t="s">
-        <v>127</v>
-      </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
+      <c r="A1" s="67" t="s">
+        <v>128</v>
+      </c>
+      <c r="B1" s="70"/>
+      <c r="C1" s="70"/>
+      <c r="D1" s="70"/>
+      <c r="E1" s="70"/>
+      <c r="F1" s="70"/>
     </row>
     <row r="3" spans="1:6" ht="13.9" customHeight="1">
-      <c r="A3" s="17" t="s">
-        <v>128</v>
-      </c>
-      <c r="B3" s="18" t="s">
+      <c r="A3" s="16" t="s">
         <v>129</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="B3" s="17" t="s">
         <v>130</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="C3" s="17" t="s">
         <v>131</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="D3" s="17" t="s">
         <v>132</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="E3" s="17" t="s">
         <v>133</v>
       </c>
+      <c r="F3" s="18" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="4" spans="1:6" ht="27" customHeight="1">
-      <c r="A4" s="12" t="s">
-        <v>134</v>
+      <c r="A4" s="11" t="s">
+        <v>135</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="F4" s="13" t="s">
         <v>139</v>
       </c>
+      <c r="F4" s="12" t="s">
+        <v>140</v>
+      </c>
     </row>
     <row r="5" spans="1:6" ht="27" customHeight="1">
-      <c r="A5" s="12" t="s">
-        <v>140</v>
+      <c r="A5" s="11" t="s">
+        <v>141</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="F5" s="13" t="s">
         <v>145</v>
       </c>
+      <c r="F5" s="12" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="6" spans="1:6" ht="27" customHeight="1">
-      <c r="A6" s="12" t="s">
-        <v>146</v>
+      <c r="A6" s="11" t="s">
+        <v>147</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="F6" s="13" t="s">
         <v>151</v>
       </c>
+      <c r="F6" s="12" t="s">
+        <v>152</v>
+      </c>
     </row>
     <row r="7" spans="1:6" ht="27" customHeight="1">
-      <c r="A7" s="12" t="s">
-        <v>152</v>
+      <c r="A7" s="11" t="s">
+        <v>153</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="F7" s="13" t="s">
         <v>157</v>
       </c>
+      <c r="F7" s="12" t="s">
+        <v>158</v>
+      </c>
     </row>
     <row r="8" spans="1:6" ht="27" customHeight="1">
-      <c r="A8" s="12" t="s">
-        <v>158</v>
+      <c r="A8" s="11" t="s">
+        <v>159</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="F8" s="13" t="s">
         <v>163</v>
       </c>
+      <c r="F8" s="12" t="s">
+        <v>164</v>
+      </c>
     </row>
     <row r="9" spans="1:6" ht="27" customHeight="1">
-      <c r="A9" s="12" t="s">
-        <v>164</v>
+      <c r="A9" s="11" t="s">
+        <v>165</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="F9" s="13" t="s">
         <v>168</v>
       </c>
+      <c r="F9" s="12" t="s">
+        <v>169</v>
+      </c>
     </row>
     <row r="10" spans="1:6" ht="27" customHeight="1">
-      <c r="A10" s="12" t="s">
-        <v>169</v>
+      <c r="A10" s="11" t="s">
+        <v>170</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="F10" s="13" t="s">
         <v>174</v>
       </c>
+      <c r="F10" s="12" t="s">
+        <v>175</v>
+      </c>
     </row>
     <row r="11" spans="1:6" ht="27" customHeight="1">
-      <c r="A11" s="20" t="s">
-        <v>175</v>
-      </c>
-      <c r="B11" s="21" t="s">
+      <c r="A11" s="19" t="s">
         <v>176</v>
       </c>
-      <c r="C11" s="21" t="s">
+      <c r="B11" s="20" t="s">
         <v>177</v>
       </c>
-      <c r="D11" s="21" t="s">
+      <c r="C11" s="20" t="s">
         <v>178</v>
       </c>
-      <c r="E11" s="21" t="s">
+      <c r="D11" s="20" t="s">
         <v>179</v>
       </c>
-      <c r="F11" s="22" t="s">
+      <c r="E11" s="20" t="s">
         <v>180</v>
       </c>
+      <c r="F11" s="21" t="s">
+        <v>181</v>
+      </c>
     </row>
     <row r="13" spans="1:6" ht="13.9" customHeight="1">
-      <c r="A13" s="72" t="s">
-        <v>181</v>
-      </c>
-      <c r="B13" s="48"/>
-      <c r="C13" s="48"/>
-      <c r="D13" s="48"/>
-      <c r="E13" s="48"/>
-      <c r="F13" s="48"/>
+      <c r="A13" s="66" t="s">
+        <v>182</v>
+      </c>
+      <c r="B13" s="70"/>
+      <c r="C13" s="70"/>
+      <c r="D13" s="70"/>
+      <c r="E13" s="70"/>
+      <c r="F13" s="70"/>
     </row>
     <row r="14" spans="1:6" ht="27" customHeight="1">
-      <c r="A14" s="23" t="s">
-        <v>182</v>
-      </c>
-      <c r="B14" s="23" t="s">
+      <c r="A14" s="22" t="s">
         <v>183</v>
       </c>
-      <c r="C14" s="23" t="s">
+      <c r="B14" s="22" t="s">
         <v>184</v>
       </c>
-      <c r="D14" s="23" t="s">
+      <c r="C14" s="22" t="s">
         <v>185</v>
       </c>
-      <c r="E14" s="23"/>
-      <c r="F14" s="23"/>
+      <c r="D14" s="22" t="s">
+        <v>186</v>
+      </c>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
     </row>
     <row r="15" spans="1:6" ht="54" customHeight="1">
-      <c r="A15" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="B15" s="23" t="s">
-        <v>186</v>
-      </c>
-      <c r="C15" s="23" t="s">
+      <c r="A15" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15" s="22" t="s">
         <v>187</v>
       </c>
-      <c r="D15" s="23" t="s">
+      <c r="C15" s="22" t="s">
         <v>188</v>
       </c>
-      <c r="E15" s="23"/>
-      <c r="F15" s="23"/>
+      <c r="D15" s="22" t="s">
+        <v>189</v>
+      </c>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2563,93 +2577,93 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="17.649999999999999" customHeight="1">
-      <c r="A1" s="74" t="s">
-        <v>189</v>
-      </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
-      <c r="J1" s="48"/>
-      <c r="K1" s="48"/>
-      <c r="L1" s="48"/>
-      <c r="M1" s="48"/>
-      <c r="N1" s="48"/>
-      <c r="O1" s="48"/>
-      <c r="P1" s="48"/>
-      <c r="Q1" s="48"/>
-      <c r="R1" s="48"/>
-      <c r="S1" s="48"/>
-      <c r="T1" s="48"/>
+      <c r="A1" s="68" t="s">
+        <v>190</v>
+      </c>
+      <c r="B1" s="70"/>
+      <c r="C1" s="70"/>
+      <c r="D1" s="70"/>
+      <c r="E1" s="70"/>
+      <c r="F1" s="70"/>
+      <c r="G1" s="70"/>
+      <c r="H1" s="70"/>
+      <c r="I1" s="70"/>
+      <c r="J1" s="70"/>
+      <c r="K1" s="70"/>
+      <c r="L1" s="70"/>
+      <c r="M1" s="70"/>
+      <c r="N1" s="70"/>
+      <c r="O1" s="70"/>
+      <c r="P1" s="70"/>
+      <c r="Q1" s="70"/>
+      <c r="R1" s="70"/>
+      <c r="S1" s="70"/>
+      <c r="T1" s="70"/>
     </row>
     <row r="3" spans="1:20" ht="13.9" customHeight="1">
-      <c r="A3" s="25" t="s">
-        <v>19</v>
-      </c>
-      <c r="B3" s="26" t="s">
+      <c r="A3" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="26" t="s">
-        <v>190</v>
-      </c>
-      <c r="D3" s="26" t="s">
-        <v>26</v>
-      </c>
-      <c r="E3" s="27">
+      <c r="B3" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" s="25" t="s">
+        <v>191</v>
+      </c>
+      <c r="D3" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="E3" s="26">
         <v>46242</v>
       </c>
-      <c r="F3" s="27">
+      <c r="F3" s="26">
         <v>46249</v>
       </c>
-      <c r="G3" s="27">
+      <c r="G3" s="26">
         <v>46256</v>
       </c>
-      <c r="H3" s="27">
+      <c r="H3" s="26">
         <v>46263</v>
       </c>
-      <c r="I3" s="27">
+      <c r="I3" s="26">
         <v>46270</v>
       </c>
-      <c r="J3" s="27">
+      <c r="J3" s="26">
         <v>46277</v>
       </c>
-      <c r="K3" s="27">
+      <c r="K3" s="26">
         <v>46284</v>
       </c>
-      <c r="L3" s="27">
+      <c r="L3" s="26">
         <v>46291</v>
       </c>
-      <c r="M3" s="27">
+      <c r="M3" s="26">
         <v>46298</v>
       </c>
-      <c r="N3" s="27">
+      <c r="N3" s="26">
         <v>46305</v>
       </c>
-      <c r="O3" s="27">
+      <c r="O3" s="26">
         <v>46312</v>
       </c>
-      <c r="P3" s="27">
+      <c r="P3" s="26">
         <v>46319</v>
       </c>
-      <c r="Q3" s="27">
+      <c r="Q3" s="26">
         <v>46326</v>
       </c>
-      <c r="R3" s="27">
+      <c r="R3" s="26">
         <v>46333</v>
       </c>
-      <c r="S3" s="27">
+      <c r="S3" s="26">
         <v>46340</v>
       </c>
-      <c r="T3" s="28">
+      <c r="T3" s="27">
         <v>46347</v>
       </c>
     </row>
     <row r="4" spans="1:20" ht="27" customHeight="1">
-      <c r="A4" s="29">
+      <c r="A4" s="28">
         <f>'Timeline tổng quan'!A13</f>
         <v>1</v>
       </c>
@@ -2665,73 +2679,73 @@
         <f>'Timeline tổng quan'!H13</f>
         <v>Hoàn thành</v>
       </c>
-      <c r="E4" s="24" t="str">
+      <c r="E4" s="23" t="str">
         <f>IF(AND(E$3&lt;='Timeline tổng quan'!$F$13,E$3+6&gt;='Timeline tổng quan'!$E$13),"■","")</f>
         <v>■</v>
       </c>
-      <c r="F4" s="24" t="str">
+      <c r="F4" s="23" t="str">
         <f>IF(AND(F$3&lt;='Timeline tổng quan'!$F$13,F$3+6&gt;='Timeline tổng quan'!$E$13),"■","")</f>
         <v/>
       </c>
-      <c r="G4" s="24" t="str">
+      <c r="G4" s="23" t="str">
         <f>IF(AND(G$3&lt;='Timeline tổng quan'!$F$13,G$3+6&gt;='Timeline tổng quan'!$E$13),"■","")</f>
         <v/>
       </c>
-      <c r="H4" s="24" t="str">
+      <c r="H4" s="23" t="str">
         <f>IF(AND(H$3&lt;='Timeline tổng quan'!$F$13,H$3+6&gt;='Timeline tổng quan'!$E$13),"■","")</f>
         <v/>
       </c>
-      <c r="I4" s="24" t="str">
+      <c r="I4" s="23" t="str">
         <f>IF(AND(I$3&lt;='Timeline tổng quan'!$F$13,I$3+6&gt;='Timeline tổng quan'!$E$13),"■","")</f>
         <v/>
       </c>
-      <c r="J4" s="24" t="str">
+      <c r="J4" s="23" t="str">
         <f>IF(AND(J$3&lt;='Timeline tổng quan'!$F$13,J$3+6&gt;='Timeline tổng quan'!$E$13),"■","")</f>
         <v/>
       </c>
-      <c r="K4" s="24" t="str">
+      <c r="K4" s="23" t="str">
         <f>IF(AND(K$3&lt;='Timeline tổng quan'!$F$13,K$3+6&gt;='Timeline tổng quan'!$E$13),"■","")</f>
         <v/>
       </c>
-      <c r="L4" s="24" t="str">
+      <c r="L4" s="23" t="str">
         <f>IF(AND(L$3&lt;='Timeline tổng quan'!$F$13,L$3+6&gt;='Timeline tổng quan'!$E$13),"■","")</f>
         <v/>
       </c>
-      <c r="M4" s="24" t="str">
+      <c r="M4" s="23" t="str">
         <f>IF(AND(M$3&lt;='Timeline tổng quan'!$F$13,M$3+6&gt;='Timeline tổng quan'!$E$13),"■","")</f>
         <v/>
       </c>
-      <c r="N4" s="24" t="str">
+      <c r="N4" s="23" t="str">
         <f>IF(AND(N$3&lt;='Timeline tổng quan'!$F$13,N$3+6&gt;='Timeline tổng quan'!$E$13),"■","")</f>
         <v/>
       </c>
-      <c r="O4" s="24" t="str">
+      <c r="O4" s="23" t="str">
         <f>IF(AND(O$3&lt;='Timeline tổng quan'!$F$13,O$3+6&gt;='Timeline tổng quan'!$E$13),"■","")</f>
         <v/>
       </c>
-      <c r="P4" s="24" t="str">
+      <c r="P4" s="23" t="str">
         <f>IF(AND(P$3&lt;='Timeline tổng quan'!$F$13,P$3+6&gt;='Timeline tổng quan'!$E$13),"■","")</f>
         <v/>
       </c>
-      <c r="Q4" s="24" t="str">
+      <c r="Q4" s="23" t="str">
         <f>IF(AND(Q$3&lt;='Timeline tổng quan'!$F$13,Q$3+6&gt;='Timeline tổng quan'!$E$13),"■","")</f>
         <v/>
       </c>
-      <c r="R4" s="24" t="str">
+      <c r="R4" s="23" t="str">
         <f>IF(AND(R$3&lt;='Timeline tổng quan'!$F$13,R$3+6&gt;='Timeline tổng quan'!$E$13),"■","")</f>
         <v/>
       </c>
-      <c r="S4" s="24" t="str">
+      <c r="S4" s="23" t="str">
         <f>IF(AND(S$3&lt;='Timeline tổng quan'!$F$13,S$3+6&gt;='Timeline tổng quan'!$E$13),"■","")</f>
         <v/>
       </c>
-      <c r="T4" s="30" t="str">
+      <c r="T4" s="29" t="str">
         <f>IF(AND(T$3&lt;='Timeline tổng quan'!$F$13,T$3+6&gt;='Timeline tổng quan'!$E$13),"■","")</f>
         <v/>
       </c>
     </row>
     <row r="5" spans="1:20" ht="27" customHeight="1">
-      <c r="A5" s="29">
+      <c r="A5" s="28">
         <f>'Timeline tổng quan'!A14</f>
         <v>2</v>
       </c>
@@ -2747,73 +2761,73 @@
         <f>'Timeline tổng quan'!H14</f>
         <v>Hoàn thành</v>
       </c>
-      <c r="E5" s="24" t="str">
+      <c r="E5" s="23" t="str">
         <f>IF(AND(E$3&lt;='Timeline tổng quan'!$F$14,E$3+6&gt;='Timeline tổng quan'!$E$14),"■","")</f>
         <v>■</v>
       </c>
-      <c r="F5" s="24" t="str">
+      <c r="F5" s="23" t="str">
         <f>IF(AND(F$3&lt;='Timeline tổng quan'!$F$14,F$3+6&gt;='Timeline tổng quan'!$E$14),"■","")</f>
         <v/>
       </c>
-      <c r="G5" s="24" t="str">
+      <c r="G5" s="23" t="str">
         <f>IF(AND(G$3&lt;='Timeline tổng quan'!$F$14,G$3+6&gt;='Timeline tổng quan'!$E$14),"■","")</f>
         <v/>
       </c>
-      <c r="H5" s="24" t="str">
+      <c r="H5" s="23" t="str">
         <f>IF(AND(H$3&lt;='Timeline tổng quan'!$F$14,H$3+6&gt;='Timeline tổng quan'!$E$14),"■","")</f>
         <v/>
       </c>
-      <c r="I5" s="24" t="str">
+      <c r="I5" s="23" t="str">
         <f>IF(AND(I$3&lt;='Timeline tổng quan'!$F$14,I$3+6&gt;='Timeline tổng quan'!$E$14),"■","")</f>
         <v/>
       </c>
-      <c r="J5" s="24" t="str">
+      <c r="J5" s="23" t="str">
         <f>IF(AND(J$3&lt;='Timeline tổng quan'!$F$14,J$3+6&gt;='Timeline tổng quan'!$E$14),"■","")</f>
         <v/>
       </c>
-      <c r="K5" s="24" t="str">
+      <c r="K5" s="23" t="str">
         <f>IF(AND(K$3&lt;='Timeline tổng quan'!$F$14,K$3+6&gt;='Timeline tổng quan'!$E$14),"■","")</f>
         <v/>
       </c>
-      <c r="L5" s="24" t="str">
+      <c r="L5" s="23" t="str">
         <f>IF(AND(L$3&lt;='Timeline tổng quan'!$F$14,L$3+6&gt;='Timeline tổng quan'!$E$14),"■","")</f>
         <v/>
       </c>
-      <c r="M5" s="24" t="str">
+      <c r="M5" s="23" t="str">
         <f>IF(AND(M$3&lt;='Timeline tổng quan'!$F$14,M$3+6&gt;='Timeline tổng quan'!$E$14),"■","")</f>
         <v/>
       </c>
-      <c r="N5" s="24" t="str">
+      <c r="N5" s="23" t="str">
         <f>IF(AND(N$3&lt;='Timeline tổng quan'!$F$14,N$3+6&gt;='Timeline tổng quan'!$E$14),"■","")</f>
         <v/>
       </c>
-      <c r="O5" s="24" t="str">
+      <c r="O5" s="23" t="str">
         <f>IF(AND(O$3&lt;='Timeline tổng quan'!$F$14,O$3+6&gt;='Timeline tổng quan'!$E$14),"■","")</f>
         <v/>
       </c>
-      <c r="P5" s="24" t="str">
+      <c r="P5" s="23" t="str">
         <f>IF(AND(P$3&lt;='Timeline tổng quan'!$F$14,P$3+6&gt;='Timeline tổng quan'!$E$14),"■","")</f>
         <v/>
       </c>
-      <c r="Q5" s="24" t="str">
+      <c r="Q5" s="23" t="str">
         <f>IF(AND(Q$3&lt;='Timeline tổng quan'!$F$14,Q$3+6&gt;='Timeline tổng quan'!$E$14),"■","")</f>
         <v/>
       </c>
-      <c r="R5" s="24" t="str">
+      <c r="R5" s="23" t="str">
         <f>IF(AND(R$3&lt;='Timeline tổng quan'!$F$14,R$3+6&gt;='Timeline tổng quan'!$E$14),"■","")</f>
         <v/>
       </c>
-      <c r="S5" s="24" t="str">
+      <c r="S5" s="23" t="str">
         <f>IF(AND(S$3&lt;='Timeline tổng quan'!$F$14,S$3+6&gt;='Timeline tổng quan'!$E$14),"■","")</f>
         <v/>
       </c>
-      <c r="T5" s="30" t="str">
+      <c r="T5" s="29" t="str">
         <f>IF(AND(T$3&lt;='Timeline tổng quan'!$F$14,T$3+6&gt;='Timeline tổng quan'!$E$14),"■","")</f>
         <v/>
       </c>
     </row>
     <row r="6" spans="1:20" ht="27" customHeight="1">
-      <c r="A6" s="29">
+      <c r="A6" s="28">
         <f>'Timeline tổng quan'!A15</f>
         <v>3</v>
       </c>
@@ -2829,73 +2843,73 @@
         <f>'Timeline tổng quan'!H15</f>
         <v>Hoàn thành</v>
       </c>
-      <c r="E6" s="24" t="str">
+      <c r="E6" s="23" t="str">
         <f>IF(AND(E$3&lt;='Timeline tổng quan'!$F$15,E$3+6&gt;='Timeline tổng quan'!$E$15),"■","")</f>
         <v>■</v>
       </c>
-      <c r="F6" s="24" t="str">
+      <c r="F6" s="23" t="str">
         <f>IF(AND(F$3&lt;='Timeline tổng quan'!$F$15,F$3+6&gt;='Timeline tổng quan'!$E$15),"■","")</f>
         <v/>
       </c>
-      <c r="G6" s="24" t="str">
+      <c r="G6" s="23" t="str">
         <f>IF(AND(G$3&lt;='Timeline tổng quan'!$F$15,G$3+6&gt;='Timeline tổng quan'!$E$15),"■","")</f>
         <v/>
       </c>
-      <c r="H6" s="24" t="str">
+      <c r="H6" s="23" t="str">
         <f>IF(AND(H$3&lt;='Timeline tổng quan'!$F$15,H$3+6&gt;='Timeline tổng quan'!$E$15),"■","")</f>
         <v/>
       </c>
-      <c r="I6" s="24" t="str">
+      <c r="I6" s="23" t="str">
         <f>IF(AND(I$3&lt;='Timeline tổng quan'!$F$15,I$3+6&gt;='Timeline tổng quan'!$E$15),"■","")</f>
         <v/>
       </c>
-      <c r="J6" s="24" t="str">
+      <c r="J6" s="23" t="str">
         <f>IF(AND(J$3&lt;='Timeline tổng quan'!$F$15,J$3+6&gt;='Timeline tổng quan'!$E$15),"■","")</f>
         <v/>
       </c>
-      <c r="K6" s="24" t="str">
+      <c r="K6" s="23" t="str">
         <f>IF(AND(K$3&lt;='Timeline tổng quan'!$F$15,K$3+6&gt;='Timeline tổng quan'!$E$15),"■","")</f>
         <v/>
       </c>
-      <c r="L6" s="24" t="str">
+      <c r="L6" s="23" t="str">
         <f>IF(AND(L$3&lt;='Timeline tổng quan'!$F$15,L$3+6&gt;='Timeline tổng quan'!$E$15),"■","")</f>
         <v/>
       </c>
-      <c r="M6" s="24" t="str">
+      <c r="M6" s="23" t="str">
         <f>IF(AND(M$3&lt;='Timeline tổng quan'!$F$15,M$3+6&gt;='Timeline tổng quan'!$E$15),"■","")</f>
         <v/>
       </c>
-      <c r="N6" s="24" t="str">
+      <c r="N6" s="23" t="str">
         <f>IF(AND(N$3&lt;='Timeline tổng quan'!$F$15,N$3+6&gt;='Timeline tổng quan'!$E$15),"■","")</f>
         <v/>
       </c>
-      <c r="O6" s="24" t="str">
+      <c r="O6" s="23" t="str">
         <f>IF(AND(O$3&lt;='Timeline tổng quan'!$F$15,O$3+6&gt;='Timeline tổng quan'!$E$15),"■","")</f>
         <v/>
       </c>
-      <c r="P6" s="24" t="str">
+      <c r="P6" s="23" t="str">
         <f>IF(AND(P$3&lt;='Timeline tổng quan'!$F$15,P$3+6&gt;='Timeline tổng quan'!$E$15),"■","")</f>
         <v/>
       </c>
-      <c r="Q6" s="24" t="str">
+      <c r="Q6" s="23" t="str">
         <f>IF(AND(Q$3&lt;='Timeline tổng quan'!$F$15,Q$3+6&gt;='Timeline tổng quan'!$E$15),"■","")</f>
         <v/>
       </c>
-      <c r="R6" s="24" t="str">
+      <c r="R6" s="23" t="str">
         <f>IF(AND(R$3&lt;='Timeline tổng quan'!$F$15,R$3+6&gt;='Timeline tổng quan'!$E$15),"■","")</f>
         <v/>
       </c>
-      <c r="S6" s="24" t="str">
+      <c r="S6" s="23" t="str">
         <f>IF(AND(S$3&lt;='Timeline tổng quan'!$F$15,S$3+6&gt;='Timeline tổng quan'!$E$15),"■","")</f>
         <v/>
       </c>
-      <c r="T6" s="30" t="str">
+      <c r="T6" s="29" t="str">
         <f>IF(AND(T$3&lt;='Timeline tổng quan'!$F$15,T$3+6&gt;='Timeline tổng quan'!$E$15),"■","")</f>
         <v/>
       </c>
     </row>
     <row r="7" spans="1:20" ht="27" customHeight="1">
-      <c r="A7" s="29">
+      <c r="A7" s="28">
         <f>'Timeline tổng quan'!A16</f>
         <v>4</v>
       </c>
@@ -2911,73 +2925,73 @@
         <f>'Timeline tổng quan'!H16</f>
         <v>Hoàn thành</v>
       </c>
-      <c r="E7" s="24" t="str">
+      <c r="E7" s="23" t="str">
         <f>IF(AND(E$3&lt;='Timeline tổng quan'!$F$16,E$3+6&gt;='Timeline tổng quan'!$E$16),"■","")</f>
         <v>■</v>
       </c>
-      <c r="F7" s="24" t="str">
+      <c r="F7" s="23" t="str">
         <f>IF(AND(F$3&lt;='Timeline tổng quan'!$F$16,F$3+6&gt;='Timeline tổng quan'!$E$16),"■","")</f>
         <v/>
       </c>
-      <c r="G7" s="24" t="str">
+      <c r="G7" s="23" t="str">
         <f>IF(AND(G$3&lt;='Timeline tổng quan'!$F$16,G$3+6&gt;='Timeline tổng quan'!$E$16),"■","")</f>
         <v/>
       </c>
-      <c r="H7" s="24" t="str">
+      <c r="H7" s="23" t="str">
         <f>IF(AND(H$3&lt;='Timeline tổng quan'!$F$16,H$3+6&gt;='Timeline tổng quan'!$E$16),"■","")</f>
         <v/>
       </c>
-      <c r="I7" s="24" t="str">
+      <c r="I7" s="23" t="str">
         <f>IF(AND(I$3&lt;='Timeline tổng quan'!$F$16,I$3+6&gt;='Timeline tổng quan'!$E$16),"■","")</f>
         <v/>
       </c>
-      <c r="J7" s="24" t="str">
+      <c r="J7" s="23" t="str">
         <f>IF(AND(J$3&lt;='Timeline tổng quan'!$F$16,J$3+6&gt;='Timeline tổng quan'!$E$16),"■","")</f>
         <v/>
       </c>
-      <c r="K7" s="24" t="str">
+      <c r="K7" s="23" t="str">
         <f>IF(AND(K$3&lt;='Timeline tổng quan'!$F$16,K$3+6&gt;='Timeline tổng quan'!$E$16),"■","")</f>
         <v/>
       </c>
-      <c r="L7" s="24" t="str">
+      <c r="L7" s="23" t="str">
         <f>IF(AND(L$3&lt;='Timeline tổng quan'!$F$16,L$3+6&gt;='Timeline tổng quan'!$E$16),"■","")</f>
         <v/>
       </c>
-      <c r="M7" s="24" t="str">
+      <c r="M7" s="23" t="str">
         <f>IF(AND(M$3&lt;='Timeline tổng quan'!$F$16,M$3+6&gt;='Timeline tổng quan'!$E$16),"■","")</f>
         <v/>
       </c>
-      <c r="N7" s="24" t="str">
+      <c r="N7" s="23" t="str">
         <f>IF(AND(N$3&lt;='Timeline tổng quan'!$F$16,N$3+6&gt;='Timeline tổng quan'!$E$16),"■","")</f>
         <v/>
       </c>
-      <c r="O7" s="24" t="str">
+      <c r="O7" s="23" t="str">
         <f>IF(AND(O$3&lt;='Timeline tổng quan'!$F$16,O$3+6&gt;='Timeline tổng quan'!$E$16),"■","")</f>
         <v/>
       </c>
-      <c r="P7" s="24" t="str">
+      <c r="P7" s="23" t="str">
         <f>IF(AND(P$3&lt;='Timeline tổng quan'!$F$16,P$3+6&gt;='Timeline tổng quan'!$E$16),"■","")</f>
         <v/>
       </c>
-      <c r="Q7" s="24" t="str">
+      <c r="Q7" s="23" t="str">
         <f>IF(AND(Q$3&lt;='Timeline tổng quan'!$F$16,Q$3+6&gt;='Timeline tổng quan'!$E$16),"■","")</f>
         <v/>
       </c>
-      <c r="R7" s="24" t="str">
+      <c r="R7" s="23" t="str">
         <f>IF(AND(R$3&lt;='Timeline tổng quan'!$F$16,R$3+6&gt;='Timeline tổng quan'!$E$16),"■","")</f>
         <v/>
       </c>
-      <c r="S7" s="24" t="str">
+      <c r="S7" s="23" t="str">
         <f>IF(AND(S$3&lt;='Timeline tổng quan'!$F$16,S$3+6&gt;='Timeline tổng quan'!$E$16),"■","")</f>
         <v/>
       </c>
-      <c r="T7" s="30" t="str">
+      <c r="T7" s="29" t="str">
         <f>IF(AND(T$3&lt;='Timeline tổng quan'!$F$16,T$3+6&gt;='Timeline tổng quan'!$E$16),"■","")</f>
         <v/>
       </c>
     </row>
     <row r="8" spans="1:20" ht="27" customHeight="1">
-      <c r="A8" s="29">
+      <c r="A8" s="28">
         <f>'Timeline tổng quan'!A17</f>
         <v>5</v>
       </c>
@@ -2993,73 +3007,73 @@
         <f>'Timeline tổng quan'!H17</f>
         <v>Hoàn thành</v>
       </c>
-      <c r="E8" s="24" t="str">
+      <c r="E8" s="23" t="str">
         <f>IF(AND(E$3&lt;='Timeline tổng quan'!$F$17,E$3+6&gt;='Timeline tổng quan'!$E$17),"■","")</f>
         <v>■</v>
       </c>
-      <c r="F8" s="24" t="str">
+      <c r="F8" s="23" t="str">
         <f>IF(AND(F$3&lt;='Timeline tổng quan'!$F$17,F$3+6&gt;='Timeline tổng quan'!$E$17),"■","")</f>
         <v/>
       </c>
-      <c r="G8" s="24" t="str">
+      <c r="G8" s="23" t="str">
         <f>IF(AND(G$3&lt;='Timeline tổng quan'!$F$17,G$3+6&gt;='Timeline tổng quan'!$E$17),"■","")</f>
         <v/>
       </c>
-      <c r="H8" s="24" t="str">
+      <c r="H8" s="23" t="str">
         <f>IF(AND(H$3&lt;='Timeline tổng quan'!$F$17,H$3+6&gt;='Timeline tổng quan'!$E$17),"■","")</f>
         <v/>
       </c>
-      <c r="I8" s="24" t="str">
+      <c r="I8" s="23" t="str">
         <f>IF(AND(I$3&lt;='Timeline tổng quan'!$F$17,I$3+6&gt;='Timeline tổng quan'!$E$17),"■","")</f>
         <v/>
       </c>
-      <c r="J8" s="24" t="str">
+      <c r="J8" s="23" t="str">
         <f>IF(AND(J$3&lt;='Timeline tổng quan'!$F$17,J$3+6&gt;='Timeline tổng quan'!$E$17),"■","")</f>
         <v/>
       </c>
-      <c r="K8" s="24" t="str">
+      <c r="K8" s="23" t="str">
         <f>IF(AND(K$3&lt;='Timeline tổng quan'!$F$17,K$3+6&gt;='Timeline tổng quan'!$E$17),"■","")</f>
         <v/>
       </c>
-      <c r="L8" s="24" t="str">
+      <c r="L8" s="23" t="str">
         <f>IF(AND(L$3&lt;='Timeline tổng quan'!$F$17,L$3+6&gt;='Timeline tổng quan'!$E$17),"■","")</f>
         <v/>
       </c>
-      <c r="M8" s="24" t="str">
+      <c r="M8" s="23" t="str">
         <f>IF(AND(M$3&lt;='Timeline tổng quan'!$F$17,M$3+6&gt;='Timeline tổng quan'!$E$17),"■","")</f>
         <v/>
       </c>
-      <c r="N8" s="24" t="str">
+      <c r="N8" s="23" t="str">
         <f>IF(AND(N$3&lt;='Timeline tổng quan'!$F$17,N$3+6&gt;='Timeline tổng quan'!$E$17),"■","")</f>
         <v/>
       </c>
-      <c r="O8" s="24" t="str">
+      <c r="O8" s="23" t="str">
         <f>IF(AND(O$3&lt;='Timeline tổng quan'!$F$17,O$3+6&gt;='Timeline tổng quan'!$E$17),"■","")</f>
         <v/>
       </c>
-      <c r="P8" s="24" t="str">
+      <c r="P8" s="23" t="str">
         <f>IF(AND(P$3&lt;='Timeline tổng quan'!$F$17,P$3+6&gt;='Timeline tổng quan'!$E$17),"■","")</f>
         <v/>
       </c>
-      <c r="Q8" s="24" t="str">
+      <c r="Q8" s="23" t="str">
         <f>IF(AND(Q$3&lt;='Timeline tổng quan'!$F$17,Q$3+6&gt;='Timeline tổng quan'!$E$17),"■","")</f>
         <v/>
       </c>
-      <c r="R8" s="24" t="str">
+      <c r="R8" s="23" t="str">
         <f>IF(AND(R$3&lt;='Timeline tổng quan'!$F$17,R$3+6&gt;='Timeline tổng quan'!$E$17),"■","")</f>
         <v/>
       </c>
-      <c r="S8" s="24" t="str">
+      <c r="S8" s="23" t="str">
         <f>IF(AND(S$3&lt;='Timeline tổng quan'!$F$17,S$3+6&gt;='Timeline tổng quan'!$E$17),"■","")</f>
         <v/>
       </c>
-      <c r="T8" s="30" t="str">
+      <c r="T8" s="29" t="str">
         <f>IF(AND(T$3&lt;='Timeline tổng quan'!$F$17,T$3+6&gt;='Timeline tổng quan'!$E$17),"■","")</f>
         <v/>
       </c>
     </row>
     <row r="9" spans="1:20" ht="13.9" customHeight="1">
-      <c r="A9" s="29">
+      <c r="A9" s="28">
         <f>'Timeline tổng quan'!A18</f>
         <v>6</v>
       </c>
@@ -3075,73 +3089,73 @@
         <f>'Timeline tổng quan'!H18</f>
         <v>Hoàn thành</v>
       </c>
-      <c r="E9" s="24" t="str">
+      <c r="E9" s="23" t="str">
         <f>IF(AND(E$3&lt;='Timeline tổng quan'!$F$18,E$3+6&gt;='Timeline tổng quan'!$E$18),"■","")</f>
         <v>■</v>
       </c>
-      <c r="F9" s="24" t="str">
+      <c r="F9" s="23" t="str">
         <f>IF(AND(F$3&lt;='Timeline tổng quan'!$F$18,F$3+6&gt;='Timeline tổng quan'!$E$18),"■","")</f>
         <v/>
       </c>
-      <c r="G9" s="24" t="str">
+      <c r="G9" s="23" t="str">
         <f>IF(AND(G$3&lt;='Timeline tổng quan'!$F$18,G$3+6&gt;='Timeline tổng quan'!$E$18),"■","")</f>
         <v/>
       </c>
-      <c r="H9" s="24" t="str">
+      <c r="H9" s="23" t="str">
         <f>IF(AND(H$3&lt;='Timeline tổng quan'!$F$18,H$3+6&gt;='Timeline tổng quan'!$E$18),"■","")</f>
         <v/>
       </c>
-      <c r="I9" s="24" t="str">
+      <c r="I9" s="23" t="str">
         <f>IF(AND(I$3&lt;='Timeline tổng quan'!$F$18,I$3+6&gt;='Timeline tổng quan'!$E$18),"■","")</f>
         <v/>
       </c>
-      <c r="J9" s="24" t="str">
+      <c r="J9" s="23" t="str">
         <f>IF(AND(J$3&lt;='Timeline tổng quan'!$F$18,J$3+6&gt;='Timeline tổng quan'!$E$18),"■","")</f>
         <v/>
       </c>
-      <c r="K9" s="24" t="str">
+      <c r="K9" s="23" t="str">
         <f>IF(AND(K$3&lt;='Timeline tổng quan'!$F$18,K$3+6&gt;='Timeline tổng quan'!$E$18),"■","")</f>
         <v/>
       </c>
-      <c r="L9" s="24" t="str">
+      <c r="L9" s="23" t="str">
         <f>IF(AND(L$3&lt;='Timeline tổng quan'!$F$18,L$3+6&gt;='Timeline tổng quan'!$E$18),"■","")</f>
         <v/>
       </c>
-      <c r="M9" s="24" t="str">
+      <c r="M9" s="23" t="str">
         <f>IF(AND(M$3&lt;='Timeline tổng quan'!$F$18,M$3+6&gt;='Timeline tổng quan'!$E$18),"■","")</f>
         <v/>
       </c>
-      <c r="N9" s="24" t="str">
+      <c r="N9" s="23" t="str">
         <f>IF(AND(N$3&lt;='Timeline tổng quan'!$F$18,N$3+6&gt;='Timeline tổng quan'!$E$18),"■","")</f>
         <v/>
       </c>
-      <c r="O9" s="24" t="str">
+      <c r="O9" s="23" t="str">
         <f>IF(AND(O$3&lt;='Timeline tổng quan'!$F$18,O$3+6&gt;='Timeline tổng quan'!$E$18),"■","")</f>
         <v/>
       </c>
-      <c r="P9" s="24" t="str">
+      <c r="P9" s="23" t="str">
         <f>IF(AND(P$3&lt;='Timeline tổng quan'!$F$18,P$3+6&gt;='Timeline tổng quan'!$E$18),"■","")</f>
         <v/>
       </c>
-      <c r="Q9" s="24" t="str">
+      <c r="Q9" s="23" t="str">
         <f>IF(AND(Q$3&lt;='Timeline tổng quan'!$F$18,Q$3+6&gt;='Timeline tổng quan'!$E$18),"■","")</f>
         <v/>
       </c>
-      <c r="R9" s="24" t="str">
+      <c r="R9" s="23" t="str">
         <f>IF(AND(R$3&lt;='Timeline tổng quan'!$F$18,R$3+6&gt;='Timeline tổng quan'!$E$18),"■","")</f>
         <v/>
       </c>
-      <c r="S9" s="24" t="str">
+      <c r="S9" s="23" t="str">
         <f>IF(AND(S$3&lt;='Timeline tổng quan'!$F$18,S$3+6&gt;='Timeline tổng quan'!$E$18),"■","")</f>
         <v/>
       </c>
-      <c r="T9" s="30" t="str">
+      <c r="T9" s="29" t="str">
         <f>IF(AND(T$3&lt;='Timeline tổng quan'!$F$18,T$3+6&gt;='Timeline tổng quan'!$E$18),"■","")</f>
         <v/>
       </c>
     </row>
     <row r="10" spans="1:20" ht="13.9" customHeight="1">
-      <c r="A10" s="29">
+      <c r="A10" s="28">
         <f>'Timeline tổng quan'!A19</f>
         <v>7</v>
       </c>
@@ -3157,73 +3171,73 @@
         <f>'Timeline tổng quan'!H19</f>
         <v>Chưa bắt đầu</v>
       </c>
-      <c r="E10" s="24" t="str">
+      <c r="E10" s="23" t="str">
         <f>IF(AND(E$3&lt;='Timeline tổng quan'!$F$19,E$3+6&gt;='Timeline tổng quan'!$E$19),"■","")</f>
         <v/>
       </c>
-      <c r="F10" s="24" t="str">
+      <c r="F10" s="23" t="str">
         <f>IF(AND(F$3&lt;='Timeline tổng quan'!$F$19,F$3+6&gt;='Timeline tổng quan'!$E$19),"■","")</f>
         <v/>
       </c>
-      <c r="G10" s="24" t="str">
+      <c r="G10" s="23" t="str">
         <f>IF(AND(G$3&lt;='Timeline tổng quan'!$F$19,G$3+6&gt;='Timeline tổng quan'!$E$19),"■","")</f>
         <v>■</v>
       </c>
-      <c r="H10" s="24" t="str">
+      <c r="H10" s="23" t="str">
         <f>IF(AND(H$3&lt;='Timeline tổng quan'!$F$19,H$3+6&gt;='Timeline tổng quan'!$E$19),"■","")</f>
         <v>■</v>
       </c>
-      <c r="I10" s="24" t="str">
+      <c r="I10" s="23" t="str">
         <f>IF(AND(I$3&lt;='Timeline tổng quan'!$F$19,I$3+6&gt;='Timeline tổng quan'!$E$19),"■","")</f>
         <v>■</v>
       </c>
-      <c r="J10" s="24" t="str">
+      <c r="J10" s="23" t="str">
         <f>IF(AND(J$3&lt;='Timeline tổng quan'!$F$19,J$3+6&gt;='Timeline tổng quan'!$E$19),"■","")</f>
         <v/>
       </c>
-      <c r="K10" s="24" t="str">
+      <c r="K10" s="23" t="str">
         <f>IF(AND(K$3&lt;='Timeline tổng quan'!$F$19,K$3+6&gt;='Timeline tổng quan'!$E$19),"■","")</f>
         <v/>
       </c>
-      <c r="L10" s="24" t="str">
+      <c r="L10" s="23" t="str">
         <f>IF(AND(L$3&lt;='Timeline tổng quan'!$F$19,L$3+6&gt;='Timeline tổng quan'!$E$19),"■","")</f>
         <v/>
       </c>
-      <c r="M10" s="24" t="str">
+      <c r="M10" s="23" t="str">
         <f>IF(AND(M$3&lt;='Timeline tổng quan'!$F$19,M$3+6&gt;='Timeline tổng quan'!$E$19),"■","")</f>
         <v/>
       </c>
-      <c r="N10" s="24" t="str">
+      <c r="N10" s="23" t="str">
         <f>IF(AND(N$3&lt;='Timeline tổng quan'!$F$19,N$3+6&gt;='Timeline tổng quan'!$E$19),"■","")</f>
         <v/>
       </c>
-      <c r="O10" s="24" t="str">
+      <c r="O10" s="23" t="str">
         <f>IF(AND(O$3&lt;='Timeline tổng quan'!$F$19,O$3+6&gt;='Timeline tổng quan'!$E$19),"■","")</f>
         <v/>
       </c>
-      <c r="P10" s="24" t="str">
+      <c r="P10" s="23" t="str">
         <f>IF(AND(P$3&lt;='Timeline tổng quan'!$F$19,P$3+6&gt;='Timeline tổng quan'!$E$19),"■","")</f>
         <v/>
       </c>
-      <c r="Q10" s="24" t="str">
+      <c r="Q10" s="23" t="str">
         <f>IF(AND(Q$3&lt;='Timeline tổng quan'!$F$19,Q$3+6&gt;='Timeline tổng quan'!$E$19),"■","")</f>
         <v/>
       </c>
-      <c r="R10" s="24" t="str">
+      <c r="R10" s="23" t="str">
         <f>IF(AND(R$3&lt;='Timeline tổng quan'!$F$19,R$3+6&gt;='Timeline tổng quan'!$E$19),"■","")</f>
         <v/>
       </c>
-      <c r="S10" s="24" t="str">
+      <c r="S10" s="23" t="str">
         <f>IF(AND(S$3&lt;='Timeline tổng quan'!$F$19,S$3+6&gt;='Timeline tổng quan'!$E$19),"■","")</f>
         <v/>
       </c>
-      <c r="T10" s="30" t="str">
+      <c r="T10" s="29" t="str">
         <f>IF(AND(T$3&lt;='Timeline tổng quan'!$F$19,T$3+6&gt;='Timeline tổng quan'!$E$19),"■","")</f>
         <v/>
       </c>
     </row>
     <row r="11" spans="1:20" ht="13.9" customHeight="1">
-      <c r="A11" s="29">
+      <c r="A11" s="28">
         <f>'Timeline tổng quan'!A20</f>
         <v>8</v>
       </c>
@@ -3239,73 +3253,73 @@
         <f>'Timeline tổng quan'!H20</f>
         <v>Hoàn thành</v>
       </c>
-      <c r="E11" s="24" t="str">
+      <c r="E11" s="23" t="str">
         <f>IF(AND(E$3&lt;='Timeline tổng quan'!$F$20,E$3+6&gt;='Timeline tổng quan'!$E$20),"■","")</f>
         <v>■</v>
       </c>
-      <c r="F11" s="24" t="str">
+      <c r="F11" s="23" t="str">
         <f>IF(AND(F$3&lt;='Timeline tổng quan'!$F$20,F$3+6&gt;='Timeline tổng quan'!$E$20),"■","")</f>
         <v/>
       </c>
-      <c r="G11" s="24" t="str">
+      <c r="G11" s="23" t="str">
         <f>IF(AND(G$3&lt;='Timeline tổng quan'!$F$20,G$3+6&gt;='Timeline tổng quan'!$E$20),"■","")</f>
         <v/>
       </c>
-      <c r="H11" s="24" t="str">
+      <c r="H11" s="23" t="str">
         <f>IF(AND(H$3&lt;='Timeline tổng quan'!$F$20,H$3+6&gt;='Timeline tổng quan'!$E$20),"■","")</f>
         <v/>
       </c>
-      <c r="I11" s="24" t="str">
+      <c r="I11" s="23" t="str">
         <f>IF(AND(I$3&lt;='Timeline tổng quan'!$F$20,I$3+6&gt;='Timeline tổng quan'!$E$20),"■","")</f>
         <v/>
       </c>
-      <c r="J11" s="24" t="str">
+      <c r="J11" s="23" t="str">
         <f>IF(AND(J$3&lt;='Timeline tổng quan'!$F$20,J$3+6&gt;='Timeline tổng quan'!$E$20),"■","")</f>
         <v/>
       </c>
-      <c r="K11" s="24" t="str">
+      <c r="K11" s="23" t="str">
         <f>IF(AND(K$3&lt;='Timeline tổng quan'!$F$20,K$3+6&gt;='Timeline tổng quan'!$E$20),"■","")</f>
         <v/>
       </c>
-      <c r="L11" s="24" t="str">
+      <c r="L11" s="23" t="str">
         <f>IF(AND(L$3&lt;='Timeline tổng quan'!$F$20,L$3+6&gt;='Timeline tổng quan'!$E$20),"■","")</f>
         <v/>
       </c>
-      <c r="M11" s="24" t="str">
+      <c r="M11" s="23" t="str">
         <f>IF(AND(M$3&lt;='Timeline tổng quan'!$F$20,M$3+6&gt;='Timeline tổng quan'!$E$20),"■","")</f>
         <v/>
       </c>
-      <c r="N11" s="24" t="str">
+      <c r="N11" s="23" t="str">
         <f>IF(AND(N$3&lt;='Timeline tổng quan'!$F$20,N$3+6&gt;='Timeline tổng quan'!$E$20),"■","")</f>
         <v/>
       </c>
-      <c r="O11" s="24" t="str">
+      <c r="O11" s="23" t="str">
         <f>IF(AND(O$3&lt;='Timeline tổng quan'!$F$20,O$3+6&gt;='Timeline tổng quan'!$E$20),"■","")</f>
         <v/>
       </c>
-      <c r="P11" s="24" t="str">
+      <c r="P11" s="23" t="str">
         <f>IF(AND(P$3&lt;='Timeline tổng quan'!$F$20,P$3+6&gt;='Timeline tổng quan'!$E$20),"■","")</f>
         <v/>
       </c>
-      <c r="Q11" s="24" t="str">
+      <c r="Q11" s="23" t="str">
         <f>IF(AND(Q$3&lt;='Timeline tổng quan'!$F$20,Q$3+6&gt;='Timeline tổng quan'!$E$20),"■","")</f>
         <v/>
       </c>
-      <c r="R11" s="24" t="str">
+      <c r="R11" s="23" t="str">
         <f>IF(AND(R$3&lt;='Timeline tổng quan'!$F$20,R$3+6&gt;='Timeline tổng quan'!$E$20),"■","")</f>
         <v/>
       </c>
-      <c r="S11" s="24" t="str">
+      <c r="S11" s="23" t="str">
         <f>IF(AND(S$3&lt;='Timeline tổng quan'!$F$20,S$3+6&gt;='Timeline tổng quan'!$E$20),"■","")</f>
         <v/>
       </c>
-      <c r="T11" s="30" t="str">
+      <c r="T11" s="29" t="str">
         <f>IF(AND(T$3&lt;='Timeline tổng quan'!$F$20,T$3+6&gt;='Timeline tổng quan'!$E$20),"■","")</f>
         <v/>
       </c>
     </row>
     <row r="12" spans="1:20" ht="27" customHeight="1">
-      <c r="A12" s="29">
+      <c r="A12" s="28">
         <f>'Timeline tổng quan'!A21</f>
         <v>9</v>
       </c>
@@ -3321,73 +3335,73 @@
         <f>'Timeline tổng quan'!H21</f>
         <v>Đang thực hiện</v>
       </c>
-      <c r="E12" s="24" t="str">
+      <c r="E12" s="23" t="str">
         <f>IF(AND(E$3&lt;='Timeline tổng quan'!$F$21,E$3+6&gt;='Timeline tổng quan'!$E$21),"■","")</f>
         <v>■</v>
       </c>
-      <c r="F12" s="24" t="str">
+      <c r="F12" s="23" t="str">
         <f>IF(AND(F$3&lt;='Timeline tổng quan'!$F$21,F$3+6&gt;='Timeline tổng quan'!$E$21),"■","")</f>
         <v>■</v>
       </c>
-      <c r="G12" s="24" t="str">
+      <c r="G12" s="23" t="str">
         <f>IF(AND(G$3&lt;='Timeline tổng quan'!$F$21,G$3+6&gt;='Timeline tổng quan'!$E$21),"■","")</f>
         <v>■</v>
       </c>
-      <c r="H12" s="24" t="str">
+      <c r="H12" s="23" t="str">
         <f>IF(AND(H$3&lt;='Timeline tổng quan'!$F$21,H$3+6&gt;='Timeline tổng quan'!$E$21),"■","")</f>
         <v>■</v>
       </c>
-      <c r="I12" s="24" t="str">
+      <c r="I12" s="23" t="str">
         <f>IF(AND(I$3&lt;='Timeline tổng quan'!$F$21,I$3+6&gt;='Timeline tổng quan'!$E$21),"■","")</f>
         <v>■</v>
       </c>
-      <c r="J12" s="24" t="str">
+      <c r="J12" s="23" t="str">
         <f>IF(AND(J$3&lt;='Timeline tổng quan'!$F$21,J$3+6&gt;='Timeline tổng quan'!$E$21),"■","")</f>
         <v>■</v>
       </c>
-      <c r="K12" s="24" t="str">
+      <c r="K12" s="23" t="str">
         <f>IF(AND(K$3&lt;='Timeline tổng quan'!$F$21,K$3+6&gt;='Timeline tổng quan'!$E$21),"■","")</f>
         <v/>
       </c>
-      <c r="L12" s="24" t="str">
+      <c r="L12" s="23" t="str">
         <f>IF(AND(L$3&lt;='Timeline tổng quan'!$F$21,L$3+6&gt;='Timeline tổng quan'!$E$21),"■","")</f>
         <v/>
       </c>
-      <c r="M12" s="24" t="str">
+      <c r="M12" s="23" t="str">
         <f>IF(AND(M$3&lt;='Timeline tổng quan'!$F$21,M$3+6&gt;='Timeline tổng quan'!$E$21),"■","")</f>
         <v/>
       </c>
-      <c r="N12" s="24" t="str">
+      <c r="N12" s="23" t="str">
         <f>IF(AND(N$3&lt;='Timeline tổng quan'!$F$21,N$3+6&gt;='Timeline tổng quan'!$E$21),"■","")</f>
         <v/>
       </c>
-      <c r="O12" s="24" t="str">
+      <c r="O12" s="23" t="str">
         <f>IF(AND(O$3&lt;='Timeline tổng quan'!$F$21,O$3+6&gt;='Timeline tổng quan'!$E$21),"■","")</f>
         <v/>
       </c>
-      <c r="P12" s="24" t="str">
+      <c r="P12" s="23" t="str">
         <f>IF(AND(P$3&lt;='Timeline tổng quan'!$F$21,P$3+6&gt;='Timeline tổng quan'!$E$21),"■","")</f>
         <v/>
       </c>
-      <c r="Q12" s="24" t="str">
+      <c r="Q12" s="23" t="str">
         <f>IF(AND(Q$3&lt;='Timeline tổng quan'!$F$21,Q$3+6&gt;='Timeline tổng quan'!$E$21),"■","")</f>
         <v/>
       </c>
-      <c r="R12" s="24" t="str">
+      <c r="R12" s="23" t="str">
         <f>IF(AND(R$3&lt;='Timeline tổng quan'!$F$21,R$3+6&gt;='Timeline tổng quan'!$E$21),"■","")</f>
         <v/>
       </c>
-      <c r="S12" s="24" t="str">
+      <c r="S12" s="23" t="str">
         <f>IF(AND(S$3&lt;='Timeline tổng quan'!$F$21,S$3+6&gt;='Timeline tổng quan'!$E$21),"■","")</f>
         <v/>
       </c>
-      <c r="T12" s="30" t="str">
+      <c r="T12" s="29" t="str">
         <f>IF(AND(T$3&lt;='Timeline tổng quan'!$F$21,T$3+6&gt;='Timeline tổng quan'!$E$21),"■","")</f>
         <v/>
       </c>
     </row>
     <row r="13" spans="1:20" ht="27" customHeight="1">
-      <c r="A13" s="29">
+      <c r="A13" s="28">
         <f>'Timeline tổng quan'!A22</f>
         <v>10</v>
       </c>
@@ -3403,73 +3417,73 @@
         <f>'Timeline tổng quan'!H22</f>
         <v>Đang thực hiện</v>
       </c>
-      <c r="E13" s="24" t="str">
+      <c r="E13" s="23" t="str">
         <f>IF(AND(E$3&lt;='Timeline tổng quan'!$F$22,E$3+6&gt;='Timeline tổng quan'!$E$22),"■","")</f>
         <v>■</v>
       </c>
-      <c r="F13" s="24" t="str">
+      <c r="F13" s="23" t="str">
         <f>IF(AND(F$3&lt;='Timeline tổng quan'!$F$22,F$3+6&gt;='Timeline tổng quan'!$E$22),"■","")</f>
         <v>■</v>
       </c>
-      <c r="G13" s="24" t="str">
+      <c r="G13" s="23" t="str">
         <f>IF(AND(G$3&lt;='Timeline tổng quan'!$F$22,G$3+6&gt;='Timeline tổng quan'!$E$22),"■","")</f>
         <v>■</v>
       </c>
-      <c r="H13" s="24" t="str">
+      <c r="H13" s="23" t="str">
         <f>IF(AND(H$3&lt;='Timeline tổng quan'!$F$22,H$3+6&gt;='Timeline tổng quan'!$E$22),"■","")</f>
         <v>■</v>
       </c>
-      <c r="I13" s="24" t="str">
+      <c r="I13" s="23" t="str">
         <f>IF(AND(I$3&lt;='Timeline tổng quan'!$F$22,I$3+6&gt;='Timeline tổng quan'!$E$22),"■","")</f>
         <v>■</v>
       </c>
-      <c r="J13" s="24" t="str">
+      <c r="J13" s="23" t="str">
         <f>IF(AND(J$3&lt;='Timeline tổng quan'!$F$22,J$3+6&gt;='Timeline tổng quan'!$E$22),"■","")</f>
         <v>■</v>
       </c>
-      <c r="K13" s="24" t="str">
+      <c r="K13" s="23" t="str">
         <f>IF(AND(K$3&lt;='Timeline tổng quan'!$F$22,K$3+6&gt;='Timeline tổng quan'!$E$22),"■","")</f>
         <v>■</v>
       </c>
-      <c r="L13" s="24" t="str">
+      <c r="L13" s="23" t="str">
         <f>IF(AND(L$3&lt;='Timeline tổng quan'!$F$22,L$3+6&gt;='Timeline tổng quan'!$E$22),"■","")</f>
         <v/>
       </c>
-      <c r="M13" s="24" t="str">
+      <c r="M13" s="23" t="str">
         <f>IF(AND(M$3&lt;='Timeline tổng quan'!$F$22,M$3+6&gt;='Timeline tổng quan'!$E$22),"■","")</f>
         <v/>
       </c>
-      <c r="N13" s="24" t="str">
+      <c r="N13" s="23" t="str">
         <f>IF(AND(N$3&lt;='Timeline tổng quan'!$F$22,N$3+6&gt;='Timeline tổng quan'!$E$22),"■","")</f>
         <v/>
       </c>
-      <c r="O13" s="24" t="str">
+      <c r="O13" s="23" t="str">
         <f>IF(AND(O$3&lt;='Timeline tổng quan'!$F$22,O$3+6&gt;='Timeline tổng quan'!$E$22),"■","")</f>
         <v/>
       </c>
-      <c r="P13" s="24" t="str">
+      <c r="P13" s="23" t="str">
         <f>IF(AND(P$3&lt;='Timeline tổng quan'!$F$22,P$3+6&gt;='Timeline tổng quan'!$E$22),"■","")</f>
         <v/>
       </c>
-      <c r="Q13" s="24" t="str">
+      <c r="Q13" s="23" t="str">
         <f>IF(AND(Q$3&lt;='Timeline tổng quan'!$F$22,Q$3+6&gt;='Timeline tổng quan'!$E$22),"■","")</f>
         <v/>
       </c>
-      <c r="R13" s="24" t="str">
+      <c r="R13" s="23" t="str">
         <f>IF(AND(R$3&lt;='Timeline tổng quan'!$F$22,R$3+6&gt;='Timeline tổng quan'!$E$22),"■","")</f>
         <v/>
       </c>
-      <c r="S13" s="24" t="str">
+      <c r="S13" s="23" t="str">
         <f>IF(AND(S$3&lt;='Timeline tổng quan'!$F$22,S$3+6&gt;='Timeline tổng quan'!$E$22),"■","")</f>
         <v/>
       </c>
-      <c r="T13" s="30" t="str">
+      <c r="T13" s="29" t="str">
         <f>IF(AND(T$3&lt;='Timeline tổng quan'!$F$22,T$3+6&gt;='Timeline tổng quan'!$E$22),"■","")</f>
         <v/>
       </c>
     </row>
     <row r="14" spans="1:20" ht="27" customHeight="1">
-      <c r="A14" s="29">
+      <c r="A14" s="28">
         <f>'Timeline tổng quan'!A23</f>
         <v>11</v>
       </c>
@@ -3485,73 +3499,73 @@
         <f>'Timeline tổng quan'!H23</f>
         <v>Chưa bắt đầu</v>
       </c>
-      <c r="E14" s="24" t="str">
+      <c r="E14" s="23" t="str">
         <f>IF(AND(E$3&lt;='Timeline tổng quan'!$F$23,E$3+6&gt;='Timeline tổng quan'!$E$23),"■","")</f>
         <v/>
       </c>
-      <c r="F14" s="24" t="str">
+      <c r="F14" s="23" t="str">
         <f>IF(AND(F$3&lt;='Timeline tổng quan'!$F$23,F$3+6&gt;='Timeline tổng quan'!$E$23),"■","")</f>
         <v/>
       </c>
-      <c r="G14" s="24" t="str">
+      <c r="G14" s="23" t="str">
         <f>IF(AND(G$3&lt;='Timeline tổng quan'!$F$23,G$3+6&gt;='Timeline tổng quan'!$E$23),"■","")</f>
         <v/>
       </c>
-      <c r="H14" s="24" t="str">
+      <c r="H14" s="23" t="str">
         <f>IF(AND(H$3&lt;='Timeline tổng quan'!$F$23,H$3+6&gt;='Timeline tổng quan'!$E$23),"■","")</f>
         <v/>
       </c>
-      <c r="I14" s="24" t="str">
+      <c r="I14" s="23" t="str">
         <f>IF(AND(I$3&lt;='Timeline tổng quan'!$F$23,I$3+6&gt;='Timeline tổng quan'!$E$23),"■","")</f>
         <v/>
       </c>
-      <c r="J14" s="24" t="str">
+      <c r="J14" s="23" t="str">
         <f>IF(AND(J$3&lt;='Timeline tổng quan'!$F$23,J$3+6&gt;='Timeline tổng quan'!$E$23),"■","")</f>
         <v/>
       </c>
-      <c r="K14" s="24" t="str">
+      <c r="K14" s="23" t="str">
         <f>IF(AND(K$3&lt;='Timeline tổng quan'!$F$23,K$3+6&gt;='Timeline tổng quan'!$E$23),"■","")</f>
         <v>■</v>
       </c>
-      <c r="L14" s="24" t="str">
+      <c r="L14" s="23" t="str">
         <f>IF(AND(L$3&lt;='Timeline tổng quan'!$F$23,L$3+6&gt;='Timeline tổng quan'!$E$23),"■","")</f>
         <v>■</v>
       </c>
-      <c r="M14" s="24" t="str">
+      <c r="M14" s="23" t="str">
         <f>IF(AND(M$3&lt;='Timeline tổng quan'!$F$23,M$3+6&gt;='Timeline tổng quan'!$E$23),"■","")</f>
         <v/>
       </c>
-      <c r="N14" s="24" t="str">
+      <c r="N14" s="23" t="str">
         <f>IF(AND(N$3&lt;='Timeline tổng quan'!$F$23,N$3+6&gt;='Timeline tổng quan'!$E$23),"■","")</f>
         <v/>
       </c>
-      <c r="O14" s="24" t="str">
+      <c r="O14" s="23" t="str">
         <f>IF(AND(O$3&lt;='Timeline tổng quan'!$F$23,O$3+6&gt;='Timeline tổng quan'!$E$23),"■","")</f>
         <v/>
       </c>
-      <c r="P14" s="24" t="str">
+      <c r="P14" s="23" t="str">
         <f>IF(AND(P$3&lt;='Timeline tổng quan'!$F$23,P$3+6&gt;='Timeline tổng quan'!$E$23),"■","")</f>
         <v/>
       </c>
-      <c r="Q14" s="24" t="str">
+      <c r="Q14" s="23" t="str">
         <f>IF(AND(Q$3&lt;='Timeline tổng quan'!$F$23,Q$3+6&gt;='Timeline tổng quan'!$E$23),"■","")</f>
         <v/>
       </c>
-      <c r="R14" s="24" t="str">
+      <c r="R14" s="23" t="str">
         <f>IF(AND(R$3&lt;='Timeline tổng quan'!$F$23,R$3+6&gt;='Timeline tổng quan'!$E$23),"■","")</f>
         <v/>
       </c>
-      <c r="S14" s="24" t="str">
+      <c r="S14" s="23" t="str">
         <f>IF(AND(S$3&lt;='Timeline tổng quan'!$F$23,S$3+6&gt;='Timeline tổng quan'!$E$23),"■","")</f>
         <v/>
       </c>
-      <c r="T14" s="30" t="str">
+      <c r="T14" s="29" t="str">
         <f>IF(AND(T$3&lt;='Timeline tổng quan'!$F$23,T$3+6&gt;='Timeline tổng quan'!$E$23),"■","")</f>
         <v/>
       </c>
     </row>
     <row r="15" spans="1:20" ht="27" customHeight="1">
-      <c r="A15" s="29">
+      <c r="A15" s="28">
         <f>'Timeline tổng quan'!A24</f>
         <v>12</v>
       </c>
@@ -3567,73 +3581,73 @@
         <f>'Timeline tổng quan'!H24</f>
         <v>Chưa bắt đầu</v>
       </c>
-      <c r="E15" s="24" t="str">
+      <c r="E15" s="23" t="str">
         <f>IF(AND(E$3&lt;='Timeline tổng quan'!$F$24,E$3+6&gt;='Timeline tổng quan'!$E$24),"■","")</f>
         <v/>
       </c>
-      <c r="F15" s="24" t="str">
+      <c r="F15" s="23" t="str">
         <f>IF(AND(F$3&lt;='Timeline tổng quan'!$F$24,F$3+6&gt;='Timeline tổng quan'!$E$24),"■","")</f>
         <v/>
       </c>
-      <c r="G15" s="24" t="str">
+      <c r="G15" s="23" t="str">
         <f>IF(AND(G$3&lt;='Timeline tổng quan'!$F$24,G$3+6&gt;='Timeline tổng quan'!$E$24),"■","")</f>
         <v/>
       </c>
-      <c r="H15" s="24" t="str">
+      <c r="H15" s="23" t="str">
         <f>IF(AND(H$3&lt;='Timeline tổng quan'!$F$24,H$3+6&gt;='Timeline tổng quan'!$E$24),"■","")</f>
         <v/>
       </c>
-      <c r="I15" s="24" t="str">
+      <c r="I15" s="23" t="str">
         <f>IF(AND(I$3&lt;='Timeline tổng quan'!$F$24,I$3+6&gt;='Timeline tổng quan'!$E$24),"■","")</f>
         <v/>
       </c>
-      <c r="J15" s="24" t="str">
+      <c r="J15" s="23" t="str">
         <f>IF(AND(J$3&lt;='Timeline tổng quan'!$F$24,J$3+6&gt;='Timeline tổng quan'!$E$24),"■","")</f>
         <v/>
       </c>
-      <c r="K15" s="24" t="str">
+      <c r="K15" s="23" t="str">
         <f>IF(AND(K$3&lt;='Timeline tổng quan'!$F$24,K$3+6&gt;='Timeline tổng quan'!$E$24),"■","")</f>
         <v/>
       </c>
-      <c r="L15" s="24" t="str">
+      <c r="L15" s="23" t="str">
         <f>IF(AND(L$3&lt;='Timeline tổng quan'!$F$24,L$3+6&gt;='Timeline tổng quan'!$E$24),"■","")</f>
         <v>■</v>
       </c>
-      <c r="M15" s="24" t="str">
+      <c r="M15" s="23" t="str">
         <f>IF(AND(M$3&lt;='Timeline tổng quan'!$F$24,M$3+6&gt;='Timeline tổng quan'!$E$24),"■","")</f>
         <v>■</v>
       </c>
-      <c r="N15" s="24" t="str">
+      <c r="N15" s="23" t="str">
         <f>IF(AND(N$3&lt;='Timeline tổng quan'!$F$24,N$3+6&gt;='Timeline tổng quan'!$E$24),"■","")</f>
         <v/>
       </c>
-      <c r="O15" s="24" t="str">
+      <c r="O15" s="23" t="str">
         <f>IF(AND(O$3&lt;='Timeline tổng quan'!$F$24,O$3+6&gt;='Timeline tổng quan'!$E$24),"■","")</f>
         <v/>
       </c>
-      <c r="P15" s="24" t="str">
+      <c r="P15" s="23" t="str">
         <f>IF(AND(P$3&lt;='Timeline tổng quan'!$F$24,P$3+6&gt;='Timeline tổng quan'!$E$24),"■","")</f>
         <v/>
       </c>
-      <c r="Q15" s="24" t="str">
+      <c r="Q15" s="23" t="str">
         <f>IF(AND(Q$3&lt;='Timeline tổng quan'!$F$24,Q$3+6&gt;='Timeline tổng quan'!$E$24),"■","")</f>
         <v/>
       </c>
-      <c r="R15" s="24" t="str">
+      <c r="R15" s="23" t="str">
         <f>IF(AND(R$3&lt;='Timeline tổng quan'!$F$24,R$3+6&gt;='Timeline tổng quan'!$E$24),"■","")</f>
         <v/>
       </c>
-      <c r="S15" s="24" t="str">
+      <c r="S15" s="23" t="str">
         <f>IF(AND(S$3&lt;='Timeline tổng quan'!$F$24,S$3+6&gt;='Timeline tổng quan'!$E$24),"■","")</f>
         <v/>
       </c>
-      <c r="T15" s="30" t="str">
+      <c r="T15" s="29" t="str">
         <f>IF(AND(T$3&lt;='Timeline tổng quan'!$F$24,T$3+6&gt;='Timeline tổng quan'!$E$24),"■","")</f>
         <v/>
       </c>
     </row>
     <row r="16" spans="1:20" ht="27" customHeight="1">
-      <c r="A16" s="29">
+      <c r="A16" s="28">
         <f>'Timeline tổng quan'!A25</f>
         <v>13</v>
       </c>
@@ -3649,73 +3663,73 @@
         <f>'Timeline tổng quan'!H25</f>
         <v>Đang thực hiện</v>
       </c>
-      <c r="E16" s="24" t="str">
+      <c r="E16" s="23" t="str">
         <f>IF(AND(E$3&lt;='Timeline tổng quan'!$F$25,E$3+6&gt;='Timeline tổng quan'!$E$25),"■","")</f>
         <v>■</v>
       </c>
-      <c r="F16" s="24" t="str">
+      <c r="F16" s="23" t="str">
         <f>IF(AND(F$3&lt;='Timeline tổng quan'!$F$25,F$3+6&gt;='Timeline tổng quan'!$E$25),"■","")</f>
         <v>■</v>
       </c>
-      <c r="G16" s="24" t="str">
+      <c r="G16" s="23" t="str">
         <f>IF(AND(G$3&lt;='Timeline tổng quan'!$F$25,G$3+6&gt;='Timeline tổng quan'!$E$25),"■","")</f>
         <v>■</v>
       </c>
-      <c r="H16" s="24" t="str">
+      <c r="H16" s="23" t="str">
         <f>IF(AND(H$3&lt;='Timeline tổng quan'!$F$25,H$3+6&gt;='Timeline tổng quan'!$E$25),"■","")</f>
         <v>■</v>
       </c>
-      <c r="I16" s="24" t="str">
+      <c r="I16" s="23" t="str">
         <f>IF(AND(I$3&lt;='Timeline tổng quan'!$F$25,I$3+6&gt;='Timeline tổng quan'!$E$25),"■","")</f>
         <v>■</v>
       </c>
-      <c r="J16" s="24" t="str">
+      <c r="J16" s="23" t="str">
         <f>IF(AND(J$3&lt;='Timeline tổng quan'!$F$25,J$3+6&gt;='Timeline tổng quan'!$E$25),"■","")</f>
         <v>■</v>
       </c>
-      <c r="K16" s="24" t="str">
+      <c r="K16" s="23" t="str">
         <f>IF(AND(K$3&lt;='Timeline tổng quan'!$F$25,K$3+6&gt;='Timeline tổng quan'!$E$25),"■","")</f>
         <v>■</v>
       </c>
-      <c r="L16" s="24" t="str">
+      <c r="L16" s="23" t="str">
         <f>IF(AND(L$3&lt;='Timeline tổng quan'!$F$25,L$3+6&gt;='Timeline tổng quan'!$E$25),"■","")</f>
         <v>■</v>
       </c>
-      <c r="M16" s="24" t="str">
+      <c r="M16" s="23" t="str">
         <f>IF(AND(M$3&lt;='Timeline tổng quan'!$F$25,M$3+6&gt;='Timeline tổng quan'!$E$25),"■","")</f>
         <v>■</v>
       </c>
-      <c r="N16" s="24" t="str">
+      <c r="N16" s="23" t="str">
         <f>IF(AND(N$3&lt;='Timeline tổng quan'!$F$25,N$3+6&gt;='Timeline tổng quan'!$E$25),"■","")</f>
         <v/>
       </c>
-      <c r="O16" s="24" t="str">
+      <c r="O16" s="23" t="str">
         <f>IF(AND(O$3&lt;='Timeline tổng quan'!$F$25,O$3+6&gt;='Timeline tổng quan'!$E$25),"■","")</f>
         <v/>
       </c>
-      <c r="P16" s="24" t="str">
+      <c r="P16" s="23" t="str">
         <f>IF(AND(P$3&lt;='Timeline tổng quan'!$F$25,P$3+6&gt;='Timeline tổng quan'!$E$25),"■","")</f>
         <v/>
       </c>
-      <c r="Q16" s="24" t="str">
+      <c r="Q16" s="23" t="str">
         <f>IF(AND(Q$3&lt;='Timeline tổng quan'!$F$25,Q$3+6&gt;='Timeline tổng quan'!$E$25),"■","")</f>
         <v/>
       </c>
-      <c r="R16" s="24" t="str">
+      <c r="R16" s="23" t="str">
         <f>IF(AND(R$3&lt;='Timeline tổng quan'!$F$25,R$3+6&gt;='Timeline tổng quan'!$E$25),"■","")</f>
         <v/>
       </c>
-      <c r="S16" s="24" t="str">
+      <c r="S16" s="23" t="str">
         <f>IF(AND(S$3&lt;='Timeline tổng quan'!$F$25,S$3+6&gt;='Timeline tổng quan'!$E$25),"■","")</f>
         <v/>
       </c>
-      <c r="T16" s="30" t="str">
+      <c r="T16" s="29" t="str">
         <f>IF(AND(T$3&lt;='Timeline tổng quan'!$F$25,T$3+6&gt;='Timeline tổng quan'!$E$25),"■","")</f>
         <v/>
       </c>
     </row>
     <row r="17" spans="1:20" ht="13.9" customHeight="1">
-      <c r="A17" s="29">
+      <c r="A17" s="28">
         <f>'Timeline tổng quan'!A26</f>
         <v>14</v>
       </c>
@@ -3731,73 +3745,73 @@
         <f>'Timeline tổng quan'!H26</f>
         <v>Chưa bắt đầu</v>
       </c>
-      <c r="E17" s="24" t="str">
+      <c r="E17" s="23" t="str">
         <f>IF(AND(E$3&lt;='Timeline tổng quan'!$F$26,E$3+6&gt;='Timeline tổng quan'!$E$26),"■","")</f>
         <v/>
       </c>
-      <c r="F17" s="24" t="str">
+      <c r="F17" s="23" t="str">
         <f>IF(AND(F$3&lt;='Timeline tổng quan'!$F$26,F$3+6&gt;='Timeline tổng quan'!$E$26),"■","")</f>
         <v/>
       </c>
-      <c r="G17" s="24" t="str">
+      <c r="G17" s="23" t="str">
         <f>IF(AND(G$3&lt;='Timeline tổng quan'!$F$26,G$3+6&gt;='Timeline tổng quan'!$E$26),"■","")</f>
         <v/>
       </c>
-      <c r="H17" s="24" t="str">
+      <c r="H17" s="23" t="str">
         <f>IF(AND(H$3&lt;='Timeline tổng quan'!$F$26,H$3+6&gt;='Timeline tổng quan'!$E$26),"■","")</f>
         <v/>
       </c>
-      <c r="I17" s="24" t="str">
+      <c r="I17" s="23" t="str">
         <f>IF(AND(I$3&lt;='Timeline tổng quan'!$F$26,I$3+6&gt;='Timeline tổng quan'!$E$26),"■","")</f>
         <v/>
       </c>
-      <c r="J17" s="24" t="str">
+      <c r="J17" s="23" t="str">
         <f>IF(AND(J$3&lt;='Timeline tổng quan'!$F$26,J$3+6&gt;='Timeline tổng quan'!$E$26),"■","")</f>
         <v/>
       </c>
-      <c r="K17" s="24" t="str">
+      <c r="K17" s="23" t="str">
         <f>IF(AND(K$3&lt;='Timeline tổng quan'!$F$26,K$3+6&gt;='Timeline tổng quan'!$E$26),"■","")</f>
         <v/>
       </c>
-      <c r="L17" s="24" t="str">
+      <c r="L17" s="23" t="str">
         <f>IF(AND(L$3&lt;='Timeline tổng quan'!$F$26,L$3+6&gt;='Timeline tổng quan'!$E$26),"■","")</f>
         <v/>
       </c>
-      <c r="M17" s="24" t="str">
+      <c r="M17" s="23" t="str">
         <f>IF(AND(M$3&lt;='Timeline tổng quan'!$F$26,M$3+6&gt;='Timeline tổng quan'!$E$26),"■","")</f>
         <v>■</v>
       </c>
-      <c r="N17" s="24" t="str">
+      <c r="N17" s="23" t="str">
         <f>IF(AND(N$3&lt;='Timeline tổng quan'!$F$26,N$3+6&gt;='Timeline tổng quan'!$E$26),"■","")</f>
         <v>■</v>
       </c>
-      <c r="O17" s="24" t="str">
+      <c r="O17" s="23" t="str">
         <f>IF(AND(O$3&lt;='Timeline tổng quan'!$F$26,O$3+6&gt;='Timeline tổng quan'!$E$26),"■","")</f>
         <v/>
       </c>
-      <c r="P17" s="24" t="str">
+      <c r="P17" s="23" t="str">
         <f>IF(AND(P$3&lt;='Timeline tổng quan'!$F$26,P$3+6&gt;='Timeline tổng quan'!$E$26),"■","")</f>
         <v/>
       </c>
-      <c r="Q17" s="24" t="str">
+      <c r="Q17" s="23" t="str">
         <f>IF(AND(Q$3&lt;='Timeline tổng quan'!$F$26,Q$3+6&gt;='Timeline tổng quan'!$E$26),"■","")</f>
         <v/>
       </c>
-      <c r="R17" s="24" t="str">
+      <c r="R17" s="23" t="str">
         <f>IF(AND(R$3&lt;='Timeline tổng quan'!$F$26,R$3+6&gt;='Timeline tổng quan'!$E$26),"■","")</f>
         <v/>
       </c>
-      <c r="S17" s="24" t="str">
+      <c r="S17" s="23" t="str">
         <f>IF(AND(S$3&lt;='Timeline tổng quan'!$F$26,S$3+6&gt;='Timeline tổng quan'!$E$26),"■","")</f>
         <v/>
       </c>
-      <c r="T17" s="30" t="str">
+      <c r="T17" s="29" t="str">
         <f>IF(AND(T$3&lt;='Timeline tổng quan'!$F$26,T$3+6&gt;='Timeline tổng quan'!$E$26),"■","")</f>
         <v/>
       </c>
     </row>
     <row r="18" spans="1:20" ht="13.9" customHeight="1">
-      <c r="A18" s="29">
+      <c r="A18" s="28">
         <f>'Timeline tổng quan'!A27</f>
         <v>15</v>
       </c>
@@ -3813,73 +3827,73 @@
         <f>'Timeline tổng quan'!H27</f>
         <v>Chưa bắt đầu</v>
       </c>
-      <c r="E18" s="24" t="str">
+      <c r="E18" s="23" t="str">
         <f>IF(AND(E$3&lt;='Timeline tổng quan'!$F$27,E$3+6&gt;='Timeline tổng quan'!$E$27),"■","")</f>
         <v/>
       </c>
-      <c r="F18" s="24" t="str">
+      <c r="F18" s="23" t="str">
         <f>IF(AND(F$3&lt;='Timeline tổng quan'!$F$27,F$3+6&gt;='Timeline tổng quan'!$E$27),"■","")</f>
         <v/>
       </c>
-      <c r="G18" s="24" t="str">
+      <c r="G18" s="23" t="str">
         <f>IF(AND(G$3&lt;='Timeline tổng quan'!$F$27,G$3+6&gt;='Timeline tổng quan'!$E$27),"■","")</f>
         <v/>
       </c>
-      <c r="H18" s="24" t="str">
+      <c r="H18" s="23" t="str">
         <f>IF(AND(H$3&lt;='Timeline tổng quan'!$F$27,H$3+6&gt;='Timeline tổng quan'!$E$27),"■","")</f>
         <v/>
       </c>
-      <c r="I18" s="24" t="str">
+      <c r="I18" s="23" t="str">
         <f>IF(AND(I$3&lt;='Timeline tổng quan'!$F$27,I$3+6&gt;='Timeline tổng quan'!$E$27),"■","")</f>
         <v/>
       </c>
-      <c r="J18" s="24" t="str">
+      <c r="J18" s="23" t="str">
         <f>IF(AND(J$3&lt;='Timeline tổng quan'!$F$27,J$3+6&gt;='Timeline tổng quan'!$E$27),"■","")</f>
         <v/>
       </c>
-      <c r="K18" s="24" t="str">
+      <c r="K18" s="23" t="str">
         <f>IF(AND(K$3&lt;='Timeline tổng quan'!$F$27,K$3+6&gt;='Timeline tổng quan'!$E$27),"■","")</f>
         <v/>
       </c>
-      <c r="L18" s="24" t="str">
+      <c r="L18" s="23" t="str">
         <f>IF(AND(L$3&lt;='Timeline tổng quan'!$F$27,L$3+6&gt;='Timeline tổng quan'!$E$27),"■","")</f>
         <v/>
       </c>
-      <c r="M18" s="24" t="str">
+      <c r="M18" s="23" t="str">
         <f>IF(AND(M$3&lt;='Timeline tổng quan'!$F$27,M$3+6&gt;='Timeline tổng quan'!$E$27),"■","")</f>
         <v/>
       </c>
-      <c r="N18" s="24" t="str">
+      <c r="N18" s="23" t="str">
         <f>IF(AND(N$3&lt;='Timeline tổng quan'!$F$27,N$3+6&gt;='Timeline tổng quan'!$E$27),"■","")</f>
         <v>■</v>
       </c>
-      <c r="O18" s="24" t="str">
+      <c r="O18" s="23" t="str">
         <f>IF(AND(O$3&lt;='Timeline tổng quan'!$F$27,O$3+6&gt;='Timeline tổng quan'!$E$27),"■","")</f>
         <v>■</v>
       </c>
-      <c r="P18" s="24" t="str">
+      <c r="P18" s="23" t="str">
         <f>IF(AND(P$3&lt;='Timeline tổng quan'!$F$27,P$3+6&gt;='Timeline tổng quan'!$E$27),"■","")</f>
         <v/>
       </c>
-      <c r="Q18" s="24" t="str">
+      <c r="Q18" s="23" t="str">
         <f>IF(AND(Q$3&lt;='Timeline tổng quan'!$F$27,Q$3+6&gt;='Timeline tổng quan'!$E$27),"■","")</f>
         <v/>
       </c>
-      <c r="R18" s="24" t="str">
+      <c r="R18" s="23" t="str">
         <f>IF(AND(R$3&lt;='Timeline tổng quan'!$F$27,R$3+6&gt;='Timeline tổng quan'!$E$27),"■","")</f>
         <v/>
       </c>
-      <c r="S18" s="24" t="str">
+      <c r="S18" s="23" t="str">
         <f>IF(AND(S$3&lt;='Timeline tổng quan'!$F$27,S$3+6&gt;='Timeline tổng quan'!$E$27),"■","")</f>
         <v/>
       </c>
-      <c r="T18" s="30" t="str">
+      <c r="T18" s="29" t="str">
         <f>IF(AND(T$3&lt;='Timeline tổng quan'!$F$27,T$3+6&gt;='Timeline tổng quan'!$E$27),"■","")</f>
         <v/>
       </c>
     </row>
     <row r="19" spans="1:20" ht="13.9" customHeight="1">
-      <c r="A19" s="29">
+      <c r="A19" s="28">
         <f>'Timeline tổng quan'!A28</f>
         <v>16</v>
       </c>
@@ -3895,73 +3909,73 @@
         <f>'Timeline tổng quan'!H28</f>
         <v>Chưa bắt đầu</v>
       </c>
-      <c r="E19" s="24" t="str">
+      <c r="E19" s="23" t="str">
         <f>IF(AND(E$3&lt;='Timeline tổng quan'!$F$28,E$3+6&gt;='Timeline tổng quan'!$E$28),"■","")</f>
         <v/>
       </c>
-      <c r="F19" s="24" t="str">
+      <c r="F19" s="23" t="str">
         <f>IF(AND(F$3&lt;='Timeline tổng quan'!$F$28,F$3+6&gt;='Timeline tổng quan'!$E$28),"■","")</f>
         <v/>
       </c>
-      <c r="G19" s="24" t="str">
+      <c r="G19" s="23" t="str">
         <f>IF(AND(G$3&lt;='Timeline tổng quan'!$F$28,G$3+6&gt;='Timeline tổng quan'!$E$28),"■","")</f>
         <v/>
       </c>
-      <c r="H19" s="24" t="str">
+      <c r="H19" s="23" t="str">
         <f>IF(AND(H$3&lt;='Timeline tổng quan'!$F$28,H$3+6&gt;='Timeline tổng quan'!$E$28),"■","")</f>
         <v/>
       </c>
-      <c r="I19" s="24" t="str">
+      <c r="I19" s="23" t="str">
         <f>IF(AND(I$3&lt;='Timeline tổng quan'!$F$28,I$3+6&gt;='Timeline tổng quan'!$E$28),"■","")</f>
         <v/>
       </c>
-      <c r="J19" s="24" t="str">
+      <c r="J19" s="23" t="str">
         <f>IF(AND(J$3&lt;='Timeline tổng quan'!$F$28,J$3+6&gt;='Timeline tổng quan'!$E$28),"■","")</f>
         <v/>
       </c>
-      <c r="K19" s="24" t="str">
+      <c r="K19" s="23" t="str">
         <f>IF(AND(K$3&lt;='Timeline tổng quan'!$F$28,K$3+6&gt;='Timeline tổng quan'!$E$28),"■","")</f>
         <v/>
       </c>
-      <c r="L19" s="24" t="str">
+      <c r="L19" s="23" t="str">
         <f>IF(AND(L$3&lt;='Timeline tổng quan'!$F$28,L$3+6&gt;='Timeline tổng quan'!$E$28),"■","")</f>
         <v/>
       </c>
-      <c r="M19" s="24" t="str">
+      <c r="M19" s="23" t="str">
         <f>IF(AND(M$3&lt;='Timeline tổng quan'!$F$28,M$3+6&gt;='Timeline tổng quan'!$E$28),"■","")</f>
         <v/>
       </c>
-      <c r="N19" s="24" t="str">
+      <c r="N19" s="23" t="str">
         <f>IF(AND(N$3&lt;='Timeline tổng quan'!$F$28,N$3+6&gt;='Timeline tổng quan'!$E$28),"■","")</f>
         <v/>
       </c>
-      <c r="O19" s="24" t="str">
+      <c r="O19" s="23" t="str">
         <f>IF(AND(O$3&lt;='Timeline tổng quan'!$F$28,O$3+6&gt;='Timeline tổng quan'!$E$28),"■","")</f>
         <v>■</v>
       </c>
-      <c r="P19" s="24" t="str">
+      <c r="P19" s="23" t="str">
         <f>IF(AND(P$3&lt;='Timeline tổng quan'!$F$28,P$3+6&gt;='Timeline tổng quan'!$E$28),"■","")</f>
         <v>■</v>
       </c>
-      <c r="Q19" s="24" t="str">
+      <c r="Q19" s="23" t="str">
         <f>IF(AND(Q$3&lt;='Timeline tổng quan'!$F$28,Q$3+6&gt;='Timeline tổng quan'!$E$28),"■","")</f>
         <v/>
       </c>
-      <c r="R19" s="24" t="str">
+      <c r="R19" s="23" t="str">
         <f>IF(AND(R$3&lt;='Timeline tổng quan'!$F$28,R$3+6&gt;='Timeline tổng quan'!$E$28),"■","")</f>
         <v/>
       </c>
-      <c r="S19" s="24" t="str">
+      <c r="S19" s="23" t="str">
         <f>IF(AND(S$3&lt;='Timeline tổng quan'!$F$28,S$3+6&gt;='Timeline tổng quan'!$E$28),"■","")</f>
         <v/>
       </c>
-      <c r="T19" s="30" t="str">
+      <c r="T19" s="29" t="str">
         <f>IF(AND(T$3&lt;='Timeline tổng quan'!$F$28,T$3+6&gt;='Timeline tổng quan'!$E$28),"■","")</f>
         <v/>
       </c>
     </row>
     <row r="20" spans="1:20" ht="13.9" customHeight="1">
-      <c r="A20" s="29">
+      <c r="A20" s="28">
         <f>'Timeline tổng quan'!A29</f>
         <v>17</v>
       </c>
@@ -3977,73 +3991,73 @@
         <f>'Timeline tổng quan'!H29</f>
         <v>Chưa bắt đầu</v>
       </c>
-      <c r="E20" s="24" t="str">
+      <c r="E20" s="23" t="str">
         <f>IF(AND(E$3&lt;='Timeline tổng quan'!$F$29,E$3+6&gt;='Timeline tổng quan'!$E$29),"■","")</f>
         <v/>
       </c>
-      <c r="F20" s="24" t="str">
+      <c r="F20" s="23" t="str">
         <f>IF(AND(F$3&lt;='Timeline tổng quan'!$F$29,F$3+6&gt;='Timeline tổng quan'!$E$29),"■","")</f>
         <v/>
       </c>
-      <c r="G20" s="24" t="str">
+      <c r="G20" s="23" t="str">
         <f>IF(AND(G$3&lt;='Timeline tổng quan'!$F$29,G$3+6&gt;='Timeline tổng quan'!$E$29),"■","")</f>
         <v/>
       </c>
-      <c r="H20" s="24" t="str">
+      <c r="H20" s="23" t="str">
         <f>IF(AND(H$3&lt;='Timeline tổng quan'!$F$29,H$3+6&gt;='Timeline tổng quan'!$E$29),"■","")</f>
         <v/>
       </c>
-      <c r="I20" s="24" t="str">
+      <c r="I20" s="23" t="str">
         <f>IF(AND(I$3&lt;='Timeline tổng quan'!$F$29,I$3+6&gt;='Timeline tổng quan'!$E$29),"■","")</f>
         <v/>
       </c>
-      <c r="J20" s="24" t="str">
+      <c r="J20" s="23" t="str">
         <f>IF(AND(J$3&lt;='Timeline tổng quan'!$F$29,J$3+6&gt;='Timeline tổng quan'!$E$29),"■","")</f>
         <v/>
       </c>
-      <c r="K20" s="24" t="str">
+      <c r="K20" s="23" t="str">
         <f>IF(AND(K$3&lt;='Timeline tổng quan'!$F$29,K$3+6&gt;='Timeline tổng quan'!$E$29),"■","")</f>
         <v/>
       </c>
-      <c r="L20" s="24" t="str">
+      <c r="L20" s="23" t="str">
         <f>IF(AND(L$3&lt;='Timeline tổng quan'!$F$29,L$3+6&gt;='Timeline tổng quan'!$E$29),"■","")</f>
         <v/>
       </c>
-      <c r="M20" s="24" t="str">
+      <c r="M20" s="23" t="str">
         <f>IF(AND(M$3&lt;='Timeline tổng quan'!$F$29,M$3+6&gt;='Timeline tổng quan'!$E$29),"■","")</f>
         <v/>
       </c>
-      <c r="N20" s="24" t="str">
+      <c r="N20" s="23" t="str">
         <f>IF(AND(N$3&lt;='Timeline tổng quan'!$F$29,N$3+6&gt;='Timeline tổng quan'!$E$29),"■","")</f>
         <v/>
       </c>
-      <c r="O20" s="24" t="str">
+      <c r="O20" s="23" t="str">
         <f>IF(AND(O$3&lt;='Timeline tổng quan'!$F$29,O$3+6&gt;='Timeline tổng quan'!$E$29),"■","")</f>
         <v>■</v>
       </c>
-      <c r="P20" s="24" t="str">
+      <c r="P20" s="23" t="str">
         <f>IF(AND(P$3&lt;='Timeline tổng quan'!$F$29,P$3+6&gt;='Timeline tổng quan'!$E$29),"■","")</f>
         <v>■</v>
       </c>
-      <c r="Q20" s="24" t="str">
+      <c r="Q20" s="23" t="str">
         <f>IF(AND(Q$3&lt;='Timeline tổng quan'!$F$29,Q$3+6&gt;='Timeline tổng quan'!$E$29),"■","")</f>
         <v/>
       </c>
-      <c r="R20" s="24" t="str">
+      <c r="R20" s="23" t="str">
         <f>IF(AND(R$3&lt;='Timeline tổng quan'!$F$29,R$3+6&gt;='Timeline tổng quan'!$E$29),"■","")</f>
         <v/>
       </c>
-      <c r="S20" s="24" t="str">
+      <c r="S20" s="23" t="str">
         <f>IF(AND(S$3&lt;='Timeline tổng quan'!$F$29,S$3+6&gt;='Timeline tổng quan'!$E$29),"■","")</f>
         <v/>
       </c>
-      <c r="T20" s="30" t="str">
+      <c r="T20" s="29" t="str">
         <f>IF(AND(T$3&lt;='Timeline tổng quan'!$F$29,T$3+6&gt;='Timeline tổng quan'!$E$29),"■","")</f>
         <v/>
       </c>
     </row>
     <row r="21" spans="1:20" ht="27" customHeight="1">
-      <c r="A21" s="29">
+      <c r="A21" s="28">
         <f>'Timeline tổng quan'!A30</f>
         <v>18</v>
       </c>
@@ -4059,73 +4073,73 @@
         <f>'Timeline tổng quan'!H30</f>
         <v>Chưa bắt đầu</v>
       </c>
-      <c r="E21" s="24" t="str">
+      <c r="E21" s="23" t="str">
         <f>IF(AND(E$3&lt;='Timeline tổng quan'!$F$30,E$3+6&gt;='Timeline tổng quan'!$E$30),"■","")</f>
         <v/>
       </c>
-      <c r="F21" s="24" t="str">
+      <c r="F21" s="23" t="str">
         <f>IF(AND(F$3&lt;='Timeline tổng quan'!$F$30,F$3+6&gt;='Timeline tổng quan'!$E$30),"■","")</f>
         <v/>
       </c>
-      <c r="G21" s="24" t="str">
+      <c r="G21" s="23" t="str">
         <f>IF(AND(G$3&lt;='Timeline tổng quan'!$F$30,G$3+6&gt;='Timeline tổng quan'!$E$30),"■","")</f>
         <v/>
       </c>
-      <c r="H21" s="24" t="str">
+      <c r="H21" s="23" t="str">
         <f>IF(AND(H$3&lt;='Timeline tổng quan'!$F$30,H$3+6&gt;='Timeline tổng quan'!$E$30),"■","")</f>
         <v/>
       </c>
-      <c r="I21" s="24" t="str">
+      <c r="I21" s="23" t="str">
         <f>IF(AND(I$3&lt;='Timeline tổng quan'!$F$30,I$3+6&gt;='Timeline tổng quan'!$E$30),"■","")</f>
         <v/>
       </c>
-      <c r="J21" s="24" t="str">
+      <c r="J21" s="23" t="str">
         <f>IF(AND(J$3&lt;='Timeline tổng quan'!$F$30,J$3+6&gt;='Timeline tổng quan'!$E$30),"■","")</f>
         <v/>
       </c>
-      <c r="K21" s="24" t="str">
+      <c r="K21" s="23" t="str">
         <f>IF(AND(K$3&lt;='Timeline tổng quan'!$F$30,K$3+6&gt;='Timeline tổng quan'!$E$30),"■","")</f>
         <v/>
       </c>
-      <c r="L21" s="24" t="str">
+      <c r="L21" s="23" t="str">
         <f>IF(AND(L$3&lt;='Timeline tổng quan'!$F$30,L$3+6&gt;='Timeline tổng quan'!$E$30),"■","")</f>
         <v/>
       </c>
-      <c r="M21" s="24" t="str">
+      <c r="M21" s="23" t="str">
         <f>IF(AND(M$3&lt;='Timeline tổng quan'!$F$30,M$3+6&gt;='Timeline tổng quan'!$E$30),"■","")</f>
         <v>■</v>
       </c>
-      <c r="N21" s="24" t="str">
+      <c r="N21" s="23" t="str">
         <f>IF(AND(N$3&lt;='Timeline tổng quan'!$F$30,N$3+6&gt;='Timeline tổng quan'!$E$30),"■","")</f>
         <v>■</v>
       </c>
-      <c r="O21" s="24" t="str">
+      <c r="O21" s="23" t="str">
         <f>IF(AND(O$3&lt;='Timeline tổng quan'!$F$30,O$3+6&gt;='Timeline tổng quan'!$E$30),"■","")</f>
         <v>■</v>
       </c>
-      <c r="P21" s="24" t="str">
+      <c r="P21" s="23" t="str">
         <f>IF(AND(P$3&lt;='Timeline tổng quan'!$F$30,P$3+6&gt;='Timeline tổng quan'!$E$30),"■","")</f>
         <v/>
       </c>
-      <c r="Q21" s="24" t="str">
+      <c r="Q21" s="23" t="str">
         <f>IF(AND(Q$3&lt;='Timeline tổng quan'!$F$30,Q$3+6&gt;='Timeline tổng quan'!$E$30),"■","")</f>
         <v/>
       </c>
-      <c r="R21" s="24" t="str">
+      <c r="R21" s="23" t="str">
         <f>IF(AND(R$3&lt;='Timeline tổng quan'!$F$30,R$3+6&gt;='Timeline tổng quan'!$E$30),"■","")</f>
         <v/>
       </c>
-      <c r="S21" s="24" t="str">
+      <c r="S21" s="23" t="str">
         <f>IF(AND(S$3&lt;='Timeline tổng quan'!$F$30,S$3+6&gt;='Timeline tổng quan'!$E$30),"■","")</f>
         <v/>
       </c>
-      <c r="T21" s="30" t="str">
+      <c r="T21" s="29" t="str">
         <f>IF(AND(T$3&lt;='Timeline tổng quan'!$F$30,T$3+6&gt;='Timeline tổng quan'!$E$30),"■","")</f>
         <v/>
       </c>
     </row>
     <row r="22" spans="1:20" ht="27" customHeight="1">
-      <c r="A22" s="29">
+      <c r="A22" s="28">
         <f>'Timeline tổng quan'!A31</f>
         <v>19</v>
       </c>
@@ -4141,73 +4155,73 @@
         <f>'Timeline tổng quan'!H31</f>
         <v>Chưa bắt đầu</v>
       </c>
-      <c r="E22" s="24" t="str">
+      <c r="E22" s="23" t="str">
         <f>IF(AND(E$3&lt;='Timeline tổng quan'!$F$31,E$3+6&gt;='Timeline tổng quan'!$E$31),"■","")</f>
         <v/>
       </c>
-      <c r="F22" s="24" t="str">
+      <c r="F22" s="23" t="str">
         <f>IF(AND(F$3&lt;='Timeline tổng quan'!$F$31,F$3+6&gt;='Timeline tổng quan'!$E$31),"■","")</f>
         <v/>
       </c>
-      <c r="G22" s="24" t="str">
+      <c r="G22" s="23" t="str">
         <f>IF(AND(G$3&lt;='Timeline tổng quan'!$F$31,G$3+6&gt;='Timeline tổng quan'!$E$31),"■","")</f>
         <v/>
       </c>
-      <c r="H22" s="24" t="str">
+      <c r="H22" s="23" t="str">
         <f>IF(AND(H$3&lt;='Timeline tổng quan'!$F$31,H$3+6&gt;='Timeline tổng quan'!$E$31),"■","")</f>
         <v/>
       </c>
-      <c r="I22" s="24" t="str">
+      <c r="I22" s="23" t="str">
         <f>IF(AND(I$3&lt;='Timeline tổng quan'!$F$31,I$3+6&gt;='Timeline tổng quan'!$E$31),"■","")</f>
         <v/>
       </c>
-      <c r="J22" s="24" t="str">
+      <c r="J22" s="23" t="str">
         <f>IF(AND(J$3&lt;='Timeline tổng quan'!$F$31,J$3+6&gt;='Timeline tổng quan'!$E$31),"■","")</f>
         <v/>
       </c>
-      <c r="K22" s="24" t="str">
+      <c r="K22" s="23" t="str">
         <f>IF(AND(K$3&lt;='Timeline tổng quan'!$F$31,K$3+6&gt;='Timeline tổng quan'!$E$31),"■","")</f>
         <v/>
       </c>
-      <c r="L22" s="24" t="str">
+      <c r="L22" s="23" t="str">
         <f>IF(AND(L$3&lt;='Timeline tổng quan'!$F$31,L$3+6&gt;='Timeline tổng quan'!$E$31),"■","")</f>
         <v/>
       </c>
-      <c r="M22" s="24" t="str">
+      <c r="M22" s="23" t="str">
         <f>IF(AND(M$3&lt;='Timeline tổng quan'!$F$31,M$3+6&gt;='Timeline tổng quan'!$E$31),"■","")</f>
         <v/>
       </c>
-      <c r="N22" s="24" t="str">
+      <c r="N22" s="23" t="str">
         <f>IF(AND(N$3&lt;='Timeline tổng quan'!$F$31,N$3+6&gt;='Timeline tổng quan'!$E$31),"■","")</f>
         <v/>
       </c>
-      <c r="O22" s="24" t="str">
+      <c r="O22" s="23" t="str">
         <f>IF(AND(O$3&lt;='Timeline tổng quan'!$F$31,O$3+6&gt;='Timeline tổng quan'!$E$31),"■","")</f>
         <v>■</v>
       </c>
-      <c r="P22" s="24" t="str">
+      <c r="P22" s="23" t="str">
         <f>IF(AND(P$3&lt;='Timeline tổng quan'!$F$31,P$3+6&gt;='Timeline tổng quan'!$E$31),"■","")</f>
         <v>■</v>
       </c>
-      <c r="Q22" s="24" t="str">
+      <c r="Q22" s="23" t="str">
         <f>IF(AND(Q$3&lt;='Timeline tổng quan'!$F$31,Q$3+6&gt;='Timeline tổng quan'!$E$31),"■","")</f>
         <v/>
       </c>
-      <c r="R22" s="24" t="str">
+      <c r="R22" s="23" t="str">
         <f>IF(AND(R$3&lt;='Timeline tổng quan'!$F$31,R$3+6&gt;='Timeline tổng quan'!$E$31),"■","")</f>
         <v/>
       </c>
-      <c r="S22" s="24" t="str">
+      <c r="S22" s="23" t="str">
         <f>IF(AND(S$3&lt;='Timeline tổng quan'!$F$31,S$3+6&gt;='Timeline tổng quan'!$E$31),"■","")</f>
         <v/>
       </c>
-      <c r="T22" s="30" t="str">
+      <c r="T22" s="29" t="str">
         <f>IF(AND(T$3&lt;='Timeline tổng quan'!$F$31,T$3+6&gt;='Timeline tổng quan'!$E$31),"■","")</f>
         <v/>
       </c>
     </row>
     <row r="23" spans="1:20" ht="27" customHeight="1">
-      <c r="A23" s="29">
+      <c r="A23" s="28">
         <f>'Timeline tổng quan'!A32</f>
         <v>20</v>
       </c>
@@ -4223,73 +4237,73 @@
         <f>'Timeline tổng quan'!H32</f>
         <v>Chưa bắt đầu</v>
       </c>
-      <c r="E23" s="24" t="str">
+      <c r="E23" s="23" t="str">
         <f>IF(AND(E$3&lt;='Timeline tổng quan'!$F$32,E$3+6&gt;='Timeline tổng quan'!$E$32),"■","")</f>
         <v/>
       </c>
-      <c r="F23" s="24" t="str">
+      <c r="F23" s="23" t="str">
         <f>IF(AND(F$3&lt;='Timeline tổng quan'!$F$32,F$3+6&gt;='Timeline tổng quan'!$E$32),"■","")</f>
         <v/>
       </c>
-      <c r="G23" s="24" t="str">
+      <c r="G23" s="23" t="str">
         <f>IF(AND(G$3&lt;='Timeline tổng quan'!$F$32,G$3+6&gt;='Timeline tổng quan'!$E$32),"■","")</f>
         <v/>
       </c>
-      <c r="H23" s="24" t="str">
+      <c r="H23" s="23" t="str">
         <f>IF(AND(H$3&lt;='Timeline tổng quan'!$F$32,H$3+6&gt;='Timeline tổng quan'!$E$32),"■","")</f>
         <v/>
       </c>
-      <c r="I23" s="24" t="str">
+      <c r="I23" s="23" t="str">
         <f>IF(AND(I$3&lt;='Timeline tổng quan'!$F$32,I$3+6&gt;='Timeline tổng quan'!$E$32),"■","")</f>
         <v/>
       </c>
-      <c r="J23" s="24" t="str">
+      <c r="J23" s="23" t="str">
         <f>IF(AND(J$3&lt;='Timeline tổng quan'!$F$32,J$3+6&gt;='Timeline tổng quan'!$E$32),"■","")</f>
         <v/>
       </c>
-      <c r="K23" s="24" t="str">
+      <c r="K23" s="23" t="str">
         <f>IF(AND(K$3&lt;='Timeline tổng quan'!$F$32,K$3+6&gt;='Timeline tổng quan'!$E$32),"■","")</f>
         <v/>
       </c>
-      <c r="L23" s="24" t="str">
+      <c r="L23" s="23" t="str">
         <f>IF(AND(L$3&lt;='Timeline tổng quan'!$F$32,L$3+6&gt;='Timeline tổng quan'!$E$32),"■","")</f>
         <v/>
       </c>
-      <c r="M23" s="24" t="str">
+      <c r="M23" s="23" t="str">
         <f>IF(AND(M$3&lt;='Timeline tổng quan'!$F$32,M$3+6&gt;='Timeline tổng quan'!$E$32),"■","")</f>
         <v/>
       </c>
-      <c r="N23" s="24" t="str">
+      <c r="N23" s="23" t="str">
         <f>IF(AND(N$3&lt;='Timeline tổng quan'!$F$32,N$3+6&gt;='Timeline tổng quan'!$E$32),"■","")</f>
         <v/>
       </c>
-      <c r="O23" s="24" t="str">
+      <c r="O23" s="23" t="str">
         <f>IF(AND(O$3&lt;='Timeline tổng quan'!$F$32,O$3+6&gt;='Timeline tổng quan'!$E$32),"■","")</f>
         <v/>
       </c>
-      <c r="P23" s="24" t="str">
+      <c r="P23" s="23" t="str">
         <f>IF(AND(P$3&lt;='Timeline tổng quan'!$F$32,P$3+6&gt;='Timeline tổng quan'!$E$32),"■","")</f>
         <v>■</v>
       </c>
-      <c r="Q23" s="24" t="str">
+      <c r="Q23" s="23" t="str">
         <f>IF(AND(Q$3&lt;='Timeline tổng quan'!$F$32,Q$3+6&gt;='Timeline tổng quan'!$E$32),"■","")</f>
         <v>■</v>
       </c>
-      <c r="R23" s="24" t="str">
+      <c r="R23" s="23" t="str">
         <f>IF(AND(R$3&lt;='Timeline tổng quan'!$F$32,R$3+6&gt;='Timeline tổng quan'!$E$32),"■","")</f>
         <v/>
       </c>
-      <c r="S23" s="24" t="str">
+      <c r="S23" s="23" t="str">
         <f>IF(AND(S$3&lt;='Timeline tổng quan'!$F$32,S$3+6&gt;='Timeline tổng quan'!$E$32),"■","")</f>
         <v/>
       </c>
-      <c r="T23" s="30" t="str">
+      <c r="T23" s="29" t="str">
         <f>IF(AND(T$3&lt;='Timeline tổng quan'!$F$32,T$3+6&gt;='Timeline tổng quan'!$E$32),"■","")</f>
         <v/>
       </c>
     </row>
     <row r="24" spans="1:20" ht="27" customHeight="1">
-      <c r="A24" s="29">
+      <c r="A24" s="28">
         <f>'Timeline tổng quan'!A33</f>
         <v>21</v>
       </c>
@@ -4305,73 +4319,73 @@
         <f>'Timeline tổng quan'!H33</f>
         <v>Chưa bắt đầu</v>
       </c>
-      <c r="E24" s="24" t="str">
+      <c r="E24" s="23" t="str">
         <f>IF(AND(E$3&lt;='Timeline tổng quan'!$F$33,E$3+6&gt;='Timeline tổng quan'!$E$33),"■","")</f>
         <v/>
       </c>
-      <c r="F24" s="24" t="str">
+      <c r="F24" s="23" t="str">
         <f>IF(AND(F$3&lt;='Timeline tổng quan'!$F$33,F$3+6&gt;='Timeline tổng quan'!$E$33),"■","")</f>
         <v/>
       </c>
-      <c r="G24" s="24" t="str">
+      <c r="G24" s="23" t="str">
         <f>IF(AND(G$3&lt;='Timeline tổng quan'!$F$33,G$3+6&gt;='Timeline tổng quan'!$E$33),"■","")</f>
         <v/>
       </c>
-      <c r="H24" s="24" t="str">
+      <c r="H24" s="23" t="str">
         <f>IF(AND(H$3&lt;='Timeline tổng quan'!$F$33,H$3+6&gt;='Timeline tổng quan'!$E$33),"■","")</f>
         <v/>
       </c>
-      <c r="I24" s="24" t="str">
+      <c r="I24" s="23" t="str">
         <f>IF(AND(I$3&lt;='Timeline tổng quan'!$F$33,I$3+6&gt;='Timeline tổng quan'!$E$33),"■","")</f>
         <v/>
       </c>
-      <c r="J24" s="24" t="str">
+      <c r="J24" s="23" t="str">
         <f>IF(AND(J$3&lt;='Timeline tổng quan'!$F$33,J$3+6&gt;='Timeline tổng quan'!$E$33),"■","")</f>
         <v/>
       </c>
-      <c r="K24" s="24" t="str">
+      <c r="K24" s="23" t="str">
         <f>IF(AND(K$3&lt;='Timeline tổng quan'!$F$33,K$3+6&gt;='Timeline tổng quan'!$E$33),"■","")</f>
         <v/>
       </c>
-      <c r="L24" s="24" t="str">
+      <c r="L24" s="23" t="str">
         <f>IF(AND(L$3&lt;='Timeline tổng quan'!$F$33,L$3+6&gt;='Timeline tổng quan'!$E$33),"■","")</f>
         <v/>
       </c>
-      <c r="M24" s="24" t="str">
+      <c r="M24" s="23" t="str">
         <f>IF(AND(M$3&lt;='Timeline tổng quan'!$F$33,M$3+6&gt;='Timeline tổng quan'!$E$33),"■","")</f>
         <v/>
       </c>
-      <c r="N24" s="24" t="str">
+      <c r="N24" s="23" t="str">
         <f>IF(AND(N$3&lt;='Timeline tổng quan'!$F$33,N$3+6&gt;='Timeline tổng quan'!$E$33),"■","")</f>
         <v/>
       </c>
-      <c r="O24" s="24" t="str">
+      <c r="O24" s="23" t="str">
         <f>IF(AND(O$3&lt;='Timeline tổng quan'!$F$33,O$3+6&gt;='Timeline tổng quan'!$E$33),"■","")</f>
         <v/>
       </c>
-      <c r="P24" s="24" t="str">
+      <c r="P24" s="23" t="str">
         <f>IF(AND(P$3&lt;='Timeline tổng quan'!$F$33,P$3+6&gt;='Timeline tổng quan'!$E$33),"■","")</f>
         <v/>
       </c>
-      <c r="Q24" s="24" t="str">
+      <c r="Q24" s="23" t="str">
         <f>IF(AND(Q$3&lt;='Timeline tổng quan'!$F$33,Q$3+6&gt;='Timeline tổng quan'!$E$33),"■","")</f>
         <v>■</v>
       </c>
-      <c r="R24" s="24" t="str">
+      <c r="R24" s="23" t="str">
         <f>IF(AND(R$3&lt;='Timeline tổng quan'!$F$33,R$3+6&gt;='Timeline tổng quan'!$E$33),"■","")</f>
         <v/>
       </c>
-      <c r="S24" s="24" t="str">
+      <c r="S24" s="23" t="str">
         <f>IF(AND(S$3&lt;='Timeline tổng quan'!$F$33,S$3+6&gt;='Timeline tổng quan'!$E$33),"■","")</f>
         <v/>
       </c>
-      <c r="T24" s="30" t="str">
+      <c r="T24" s="29" t="str">
         <f>IF(AND(T$3&lt;='Timeline tổng quan'!$F$33,T$3+6&gt;='Timeline tổng quan'!$E$33),"■","")</f>
         <v/>
       </c>
     </row>
     <row r="25" spans="1:20" ht="27" customHeight="1">
-      <c r="A25" s="29">
+      <c r="A25" s="28">
         <f>'Timeline tổng quan'!A34</f>
         <v>22</v>
       </c>
@@ -4387,73 +4401,73 @@
         <f>'Timeline tổng quan'!H34</f>
         <v>Chưa bắt đầu</v>
       </c>
-      <c r="E25" s="24" t="str">
+      <c r="E25" s="23" t="str">
         <f>IF(AND(E$3&lt;='Timeline tổng quan'!$F$34,E$3+6&gt;='Timeline tổng quan'!$E$34),"■","")</f>
         <v/>
       </c>
-      <c r="F25" s="24" t="str">
+      <c r="F25" s="23" t="str">
         <f>IF(AND(F$3&lt;='Timeline tổng quan'!$F$34,F$3+6&gt;='Timeline tổng quan'!$E$34),"■","")</f>
         <v/>
       </c>
-      <c r="G25" s="24" t="str">
+      <c r="G25" s="23" t="str">
         <f>IF(AND(G$3&lt;='Timeline tổng quan'!$F$34,G$3+6&gt;='Timeline tổng quan'!$E$34),"■","")</f>
         <v/>
       </c>
-      <c r="H25" s="24" t="str">
+      <c r="H25" s="23" t="str">
         <f>IF(AND(H$3&lt;='Timeline tổng quan'!$F$34,H$3+6&gt;='Timeline tổng quan'!$E$34),"■","")</f>
         <v/>
       </c>
-      <c r="I25" s="24" t="str">
+      <c r="I25" s="23" t="str">
         <f>IF(AND(I$3&lt;='Timeline tổng quan'!$F$34,I$3+6&gt;='Timeline tổng quan'!$E$34),"■","")</f>
         <v/>
       </c>
-      <c r="J25" s="24" t="str">
+      <c r="J25" s="23" t="str">
         <f>IF(AND(J$3&lt;='Timeline tổng quan'!$F$34,J$3+6&gt;='Timeline tổng quan'!$E$34),"■","")</f>
         <v/>
       </c>
-      <c r="K25" s="24" t="str">
+      <c r="K25" s="23" t="str">
         <f>IF(AND(K$3&lt;='Timeline tổng quan'!$F$34,K$3+6&gt;='Timeline tổng quan'!$E$34),"■","")</f>
         <v/>
       </c>
-      <c r="L25" s="24" t="str">
+      <c r="L25" s="23" t="str">
         <f>IF(AND(L$3&lt;='Timeline tổng quan'!$F$34,L$3+6&gt;='Timeline tổng quan'!$E$34),"■","")</f>
         <v/>
       </c>
-      <c r="M25" s="24" t="str">
+      <c r="M25" s="23" t="str">
         <f>IF(AND(M$3&lt;='Timeline tổng quan'!$F$34,M$3+6&gt;='Timeline tổng quan'!$E$34),"■","")</f>
         <v/>
       </c>
-      <c r="N25" s="24" t="str">
+      <c r="N25" s="23" t="str">
         <f>IF(AND(N$3&lt;='Timeline tổng quan'!$F$34,N$3+6&gt;='Timeline tổng quan'!$E$34),"■","")</f>
         <v/>
       </c>
-      <c r="O25" s="24" t="str">
+      <c r="O25" s="23" t="str">
         <f>IF(AND(O$3&lt;='Timeline tổng quan'!$F$34,O$3+6&gt;='Timeline tổng quan'!$E$34),"■","")</f>
         <v/>
       </c>
-      <c r="P25" s="24" t="str">
+      <c r="P25" s="23" t="str">
         <f>IF(AND(P$3&lt;='Timeline tổng quan'!$F$34,P$3+6&gt;='Timeline tổng quan'!$E$34),"■","")</f>
         <v/>
       </c>
-      <c r="Q25" s="24" t="str">
+      <c r="Q25" s="23" t="str">
         <f>IF(AND(Q$3&lt;='Timeline tổng quan'!$F$34,Q$3+6&gt;='Timeline tổng quan'!$E$34),"■","")</f>
         <v>■</v>
       </c>
-      <c r="R25" s="24" t="str">
+      <c r="R25" s="23" t="str">
         <f>IF(AND(R$3&lt;='Timeline tổng quan'!$F$34,R$3+6&gt;='Timeline tổng quan'!$E$34),"■","")</f>
         <v/>
       </c>
-      <c r="S25" s="24" t="str">
+      <c r="S25" s="23" t="str">
         <f>IF(AND(S$3&lt;='Timeline tổng quan'!$F$34,S$3+6&gt;='Timeline tổng quan'!$E$34),"■","")</f>
         <v/>
       </c>
-      <c r="T25" s="30" t="str">
+      <c r="T25" s="29" t="str">
         <f>IF(AND(T$3&lt;='Timeline tổng quan'!$F$34,T$3+6&gt;='Timeline tổng quan'!$E$34),"■","")</f>
         <v/>
       </c>
     </row>
     <row r="26" spans="1:20" ht="27" customHeight="1">
-      <c r="A26" s="29">
+      <c r="A26" s="28">
         <f>'Timeline tổng quan'!A35</f>
         <v>23</v>
       </c>
@@ -4469,73 +4483,73 @@
         <f>'Timeline tổng quan'!H35</f>
         <v>Chưa bắt đầu</v>
       </c>
-      <c r="E26" s="24" t="str">
+      <c r="E26" s="23" t="str">
         <f>IF(AND(E$3&lt;='Timeline tổng quan'!$F$35,E$3+6&gt;='Timeline tổng quan'!$E$35),"■","")</f>
         <v/>
       </c>
-      <c r="F26" s="24" t="str">
+      <c r="F26" s="23" t="str">
         <f>IF(AND(F$3&lt;='Timeline tổng quan'!$F$35,F$3+6&gt;='Timeline tổng quan'!$E$35),"■","")</f>
         <v/>
       </c>
-      <c r="G26" s="24" t="str">
+      <c r="G26" s="23" t="str">
         <f>IF(AND(G$3&lt;='Timeline tổng quan'!$F$35,G$3+6&gt;='Timeline tổng quan'!$E$35),"■","")</f>
         <v/>
       </c>
-      <c r="H26" s="24" t="str">
+      <c r="H26" s="23" t="str">
         <f>IF(AND(H$3&lt;='Timeline tổng quan'!$F$35,H$3+6&gt;='Timeline tổng quan'!$E$35),"■","")</f>
         <v/>
       </c>
-      <c r="I26" s="24" t="str">
+      <c r="I26" s="23" t="str">
         <f>IF(AND(I$3&lt;='Timeline tổng quan'!$F$35,I$3+6&gt;='Timeline tổng quan'!$E$35),"■","")</f>
         <v/>
       </c>
-      <c r="J26" s="24" t="str">
+      <c r="J26" s="23" t="str">
         <f>IF(AND(J$3&lt;='Timeline tổng quan'!$F$35,J$3+6&gt;='Timeline tổng quan'!$E$35),"■","")</f>
         <v/>
       </c>
-      <c r="K26" s="24" t="str">
+      <c r="K26" s="23" t="str">
         <f>IF(AND(K$3&lt;='Timeline tổng quan'!$F$35,K$3+6&gt;='Timeline tổng quan'!$E$35),"■","")</f>
         <v/>
       </c>
-      <c r="L26" s="24" t="str">
+      <c r="L26" s="23" t="str">
         <f>IF(AND(L$3&lt;='Timeline tổng quan'!$F$35,L$3+6&gt;='Timeline tổng quan'!$E$35),"■","")</f>
         <v/>
       </c>
-      <c r="M26" s="24" t="str">
+      <c r="M26" s="23" t="str">
         <f>IF(AND(M$3&lt;='Timeline tổng quan'!$F$35,M$3+6&gt;='Timeline tổng quan'!$E$35),"■","")</f>
         <v/>
       </c>
-      <c r="N26" s="24" t="str">
+      <c r="N26" s="23" t="str">
         <f>IF(AND(N$3&lt;='Timeline tổng quan'!$F$35,N$3+6&gt;='Timeline tổng quan'!$E$35),"■","")</f>
         <v/>
       </c>
-      <c r="O26" s="24" t="str">
+      <c r="O26" s="23" t="str">
         <f>IF(AND(O$3&lt;='Timeline tổng quan'!$F$35,O$3+6&gt;='Timeline tổng quan'!$E$35),"■","")</f>
         <v/>
       </c>
-      <c r="P26" s="24" t="str">
+      <c r="P26" s="23" t="str">
         <f>IF(AND(P$3&lt;='Timeline tổng quan'!$F$35,P$3+6&gt;='Timeline tổng quan'!$E$35),"■","")</f>
         <v/>
       </c>
-      <c r="Q26" s="24" t="str">
+      <c r="Q26" s="23" t="str">
         <f>IF(AND(Q$3&lt;='Timeline tổng quan'!$F$35,Q$3+6&gt;='Timeline tổng quan'!$E$35),"■","")</f>
         <v/>
       </c>
-      <c r="R26" s="24" t="str">
+      <c r="R26" s="23" t="str">
         <f>IF(AND(R$3&lt;='Timeline tổng quan'!$F$35,R$3+6&gt;='Timeline tổng quan'!$E$35),"■","")</f>
         <v>■</v>
       </c>
-      <c r="S26" s="24" t="str">
+      <c r="S26" s="23" t="str">
         <f>IF(AND(S$3&lt;='Timeline tổng quan'!$F$35,S$3+6&gt;='Timeline tổng quan'!$E$35),"■","")</f>
         <v/>
       </c>
-      <c r="T26" s="30" t="str">
+      <c r="T26" s="29" t="str">
         <f>IF(AND(T$3&lt;='Timeline tổng quan'!$F$35,T$3+6&gt;='Timeline tổng quan'!$E$35),"■","")</f>
         <v/>
       </c>
     </row>
     <row r="27" spans="1:20" ht="27" customHeight="1">
-      <c r="A27" s="29">
+      <c r="A27" s="28">
         <f>'Timeline tổng quan'!A36</f>
         <v>24</v>
       </c>
@@ -4551,73 +4565,73 @@
         <f>'Timeline tổng quan'!H36</f>
         <v>Chưa bắt đầu</v>
       </c>
-      <c r="E27" s="24" t="str">
+      <c r="E27" s="23" t="str">
         <f>IF(AND(E$3&lt;='Timeline tổng quan'!$F$36,E$3+6&gt;='Timeline tổng quan'!$E$36),"■","")</f>
         <v/>
       </c>
-      <c r="F27" s="24" t="str">
+      <c r="F27" s="23" t="str">
         <f>IF(AND(F$3&lt;='Timeline tổng quan'!$F$36,F$3+6&gt;='Timeline tổng quan'!$E$36),"■","")</f>
         <v/>
       </c>
-      <c r="G27" s="24" t="str">
+      <c r="G27" s="23" t="str">
         <f>IF(AND(G$3&lt;='Timeline tổng quan'!$F$36,G$3+6&gt;='Timeline tổng quan'!$E$36),"■","")</f>
         <v/>
       </c>
-      <c r="H27" s="24" t="str">
+      <c r="H27" s="23" t="str">
         <f>IF(AND(H$3&lt;='Timeline tổng quan'!$F$36,H$3+6&gt;='Timeline tổng quan'!$E$36),"■","")</f>
         <v/>
       </c>
-      <c r="I27" s="24" t="str">
+      <c r="I27" s="23" t="str">
         <f>IF(AND(I$3&lt;='Timeline tổng quan'!$F$36,I$3+6&gt;='Timeline tổng quan'!$E$36),"■","")</f>
         <v/>
       </c>
-      <c r="J27" s="24" t="str">
+      <c r="J27" s="23" t="str">
         <f>IF(AND(J$3&lt;='Timeline tổng quan'!$F$36,J$3+6&gt;='Timeline tổng quan'!$E$36),"■","")</f>
         <v/>
       </c>
-      <c r="K27" s="24" t="str">
+      <c r="K27" s="23" t="str">
         <f>IF(AND(K$3&lt;='Timeline tổng quan'!$F$36,K$3+6&gt;='Timeline tổng quan'!$E$36),"■","")</f>
         <v/>
       </c>
-      <c r="L27" s="24" t="str">
+      <c r="L27" s="23" t="str">
         <f>IF(AND(L$3&lt;='Timeline tổng quan'!$F$36,L$3+6&gt;='Timeline tổng quan'!$E$36),"■","")</f>
         <v/>
       </c>
-      <c r="M27" s="24" t="str">
+      <c r="M27" s="23" t="str">
         <f>IF(AND(M$3&lt;='Timeline tổng quan'!$F$36,M$3+6&gt;='Timeline tổng quan'!$E$36),"■","")</f>
         <v/>
       </c>
-      <c r="N27" s="24" t="str">
+      <c r="N27" s="23" t="str">
         <f>IF(AND(N$3&lt;='Timeline tổng quan'!$F$36,N$3+6&gt;='Timeline tổng quan'!$E$36),"■","")</f>
         <v/>
       </c>
-      <c r="O27" s="24" t="str">
+      <c r="O27" s="23" t="str">
         <f>IF(AND(O$3&lt;='Timeline tổng quan'!$F$36,O$3+6&gt;='Timeline tổng quan'!$E$36),"■","")</f>
         <v/>
       </c>
-      <c r="P27" s="24" t="str">
+      <c r="P27" s="23" t="str">
         <f>IF(AND(P$3&lt;='Timeline tổng quan'!$F$36,P$3+6&gt;='Timeline tổng quan'!$E$36),"■","")</f>
         <v/>
       </c>
-      <c r="Q27" s="24" t="str">
+      <c r="Q27" s="23" t="str">
         <f>IF(AND(Q$3&lt;='Timeline tổng quan'!$F$36,Q$3+6&gt;='Timeline tổng quan'!$E$36),"■","")</f>
         <v/>
       </c>
-      <c r="R27" s="24" t="str">
+      <c r="R27" s="23" t="str">
         <f>IF(AND(R$3&lt;='Timeline tổng quan'!$F$36,R$3+6&gt;='Timeline tổng quan'!$E$36),"■","")</f>
         <v>■</v>
       </c>
-      <c r="S27" s="24" t="str">
+      <c r="S27" s="23" t="str">
         <f>IF(AND(S$3&lt;='Timeline tổng quan'!$F$36,S$3+6&gt;='Timeline tổng quan'!$E$36),"■","")</f>
         <v>■</v>
       </c>
-      <c r="T27" s="30" t="str">
+      <c r="T27" s="29" t="str">
         <f>IF(AND(T$3&lt;='Timeline tổng quan'!$F$36,T$3+6&gt;='Timeline tổng quan'!$E$36),"■","")</f>
         <v/>
       </c>
     </row>
     <row r="28" spans="1:20" ht="27" customHeight="1">
-      <c r="A28" s="29">
+      <c r="A28" s="28">
         <f>'Timeline tổng quan'!A37</f>
         <v>25</v>
       </c>
@@ -4633,73 +4647,73 @@
         <f>'Timeline tổng quan'!H37</f>
         <v>Chưa bắt đầu</v>
       </c>
-      <c r="E28" s="24" t="str">
+      <c r="E28" s="23" t="str">
         <f>IF(AND(E$3&lt;='Timeline tổng quan'!$F$37,E$3+6&gt;='Timeline tổng quan'!$E$37),"■","")</f>
         <v/>
       </c>
-      <c r="F28" s="24" t="str">
+      <c r="F28" s="23" t="str">
         <f>IF(AND(F$3&lt;='Timeline tổng quan'!$F$37,F$3+6&gt;='Timeline tổng quan'!$E$37),"■","")</f>
         <v/>
       </c>
-      <c r="G28" s="24" t="str">
+      <c r="G28" s="23" t="str">
         <f>IF(AND(G$3&lt;='Timeline tổng quan'!$F$37,G$3+6&gt;='Timeline tổng quan'!$E$37),"■","")</f>
         <v/>
       </c>
-      <c r="H28" s="24" t="str">
+      <c r="H28" s="23" t="str">
         <f>IF(AND(H$3&lt;='Timeline tổng quan'!$F$37,H$3+6&gt;='Timeline tổng quan'!$E$37),"■","")</f>
         <v/>
       </c>
-      <c r="I28" s="24" t="str">
+      <c r="I28" s="23" t="str">
         <f>IF(AND(I$3&lt;='Timeline tổng quan'!$F$37,I$3+6&gt;='Timeline tổng quan'!$E$37),"■","")</f>
         <v/>
       </c>
-      <c r="J28" s="24" t="str">
+      <c r="J28" s="23" t="str">
         <f>IF(AND(J$3&lt;='Timeline tổng quan'!$F$37,J$3+6&gt;='Timeline tổng quan'!$E$37),"■","")</f>
         <v/>
       </c>
-      <c r="K28" s="24" t="str">
+      <c r="K28" s="23" t="str">
         <f>IF(AND(K$3&lt;='Timeline tổng quan'!$F$37,K$3+6&gt;='Timeline tổng quan'!$E$37),"■","")</f>
         <v/>
       </c>
-      <c r="L28" s="24" t="str">
+      <c r="L28" s="23" t="str">
         <f>IF(AND(L$3&lt;='Timeline tổng quan'!$F$37,L$3+6&gt;='Timeline tổng quan'!$E$37),"■","")</f>
         <v/>
       </c>
-      <c r="M28" s="24" t="str">
+      <c r="M28" s="23" t="str">
         <f>IF(AND(M$3&lt;='Timeline tổng quan'!$F$37,M$3+6&gt;='Timeline tổng quan'!$E$37),"■","")</f>
         <v/>
       </c>
-      <c r="N28" s="24" t="str">
+      <c r="N28" s="23" t="str">
         <f>IF(AND(N$3&lt;='Timeline tổng quan'!$F$37,N$3+6&gt;='Timeline tổng quan'!$E$37),"■","")</f>
         <v/>
       </c>
-      <c r="O28" s="24" t="str">
+      <c r="O28" s="23" t="str">
         <f>IF(AND(O$3&lt;='Timeline tổng quan'!$F$37,O$3+6&gt;='Timeline tổng quan'!$E$37),"■","")</f>
         <v/>
       </c>
-      <c r="P28" s="24" t="str">
+      <c r="P28" s="23" t="str">
         <f>IF(AND(P$3&lt;='Timeline tổng quan'!$F$37,P$3+6&gt;='Timeline tổng quan'!$E$37),"■","")</f>
         <v/>
       </c>
-      <c r="Q28" s="24" t="str">
+      <c r="Q28" s="23" t="str">
         <f>IF(AND(Q$3&lt;='Timeline tổng quan'!$F$37,Q$3+6&gt;='Timeline tổng quan'!$E$37),"■","")</f>
         <v/>
       </c>
-      <c r="R28" s="24" t="str">
+      <c r="R28" s="23" t="str">
         <f>IF(AND(R$3&lt;='Timeline tổng quan'!$F$37,R$3+6&gt;='Timeline tổng quan'!$E$37),"■","")</f>
         <v/>
       </c>
-      <c r="S28" s="24" t="str">
+      <c r="S28" s="23" t="str">
         <f>IF(AND(S$3&lt;='Timeline tổng quan'!$F$37,S$3+6&gt;='Timeline tổng quan'!$E$37),"■","")</f>
         <v>■</v>
       </c>
-      <c r="T28" s="30" t="str">
+      <c r="T28" s="29" t="str">
         <f>IF(AND(T$3&lt;='Timeline tổng quan'!$F$37,T$3+6&gt;='Timeline tổng quan'!$E$37),"■","")</f>
         <v/>
       </c>
     </row>
     <row r="29" spans="1:20" ht="27" customHeight="1">
-      <c r="A29" s="29">
+      <c r="A29" s="28">
         <f>'Timeline tổng quan'!A38</f>
         <v>26</v>
       </c>
@@ -4715,192 +4729,192 @@
         <f>'Timeline tổng quan'!H38</f>
         <v>Chưa bắt đầu</v>
       </c>
-      <c r="E29" s="24" t="str">
+      <c r="E29" s="23" t="str">
         <f>IF(AND(E$3&lt;='Timeline tổng quan'!$F$38,E$3+6&gt;='Timeline tổng quan'!$E$38),"■","")</f>
         <v/>
       </c>
-      <c r="F29" s="24" t="str">
+      <c r="F29" s="23" t="str">
         <f>IF(AND(F$3&lt;='Timeline tổng quan'!$F$38,F$3+6&gt;='Timeline tổng quan'!$E$38),"■","")</f>
         <v/>
       </c>
-      <c r="G29" s="24" t="str">
+      <c r="G29" s="23" t="str">
         <f>IF(AND(G$3&lt;='Timeline tổng quan'!$F$38,G$3+6&gt;='Timeline tổng quan'!$E$38),"■","")</f>
         <v/>
       </c>
-      <c r="H29" s="24" t="str">
+      <c r="H29" s="23" t="str">
         <f>IF(AND(H$3&lt;='Timeline tổng quan'!$F$38,H$3+6&gt;='Timeline tổng quan'!$E$38),"■","")</f>
         <v/>
       </c>
-      <c r="I29" s="24" t="str">
+      <c r="I29" s="23" t="str">
         <f>IF(AND(I$3&lt;='Timeline tổng quan'!$F$38,I$3+6&gt;='Timeline tổng quan'!$E$38),"■","")</f>
         <v/>
       </c>
-      <c r="J29" s="24" t="str">
+      <c r="J29" s="23" t="str">
         <f>IF(AND(J$3&lt;='Timeline tổng quan'!$F$38,J$3+6&gt;='Timeline tổng quan'!$E$38),"■","")</f>
         <v/>
       </c>
-      <c r="K29" s="24" t="str">
+      <c r="K29" s="23" t="str">
         <f>IF(AND(K$3&lt;='Timeline tổng quan'!$F$38,K$3+6&gt;='Timeline tổng quan'!$E$38),"■","")</f>
         <v/>
       </c>
-      <c r="L29" s="24" t="str">
+      <c r="L29" s="23" t="str">
         <f>IF(AND(L$3&lt;='Timeline tổng quan'!$F$38,L$3+6&gt;='Timeline tổng quan'!$E$38),"■","")</f>
         <v/>
       </c>
-      <c r="M29" s="24" t="str">
+      <c r="M29" s="23" t="str">
         <f>IF(AND(M$3&lt;='Timeline tổng quan'!$F$38,M$3+6&gt;='Timeline tổng quan'!$E$38),"■","")</f>
         <v/>
       </c>
-      <c r="N29" s="24" t="str">
+      <c r="N29" s="23" t="str">
         <f>IF(AND(N$3&lt;='Timeline tổng quan'!$F$38,N$3+6&gt;='Timeline tổng quan'!$E$38),"■","")</f>
         <v/>
       </c>
-      <c r="O29" s="24" t="str">
+      <c r="O29" s="23" t="str">
         <f>IF(AND(O$3&lt;='Timeline tổng quan'!$F$38,O$3+6&gt;='Timeline tổng quan'!$E$38),"■","")</f>
         <v/>
       </c>
-      <c r="P29" s="24" t="str">
+      <c r="P29" s="23" t="str">
         <f>IF(AND(P$3&lt;='Timeline tổng quan'!$F$38,P$3+6&gt;='Timeline tổng quan'!$E$38),"■","")</f>
         <v/>
       </c>
-      <c r="Q29" s="24" t="str">
+      <c r="Q29" s="23" t="str">
         <f>IF(AND(Q$3&lt;='Timeline tổng quan'!$F$38,Q$3+6&gt;='Timeline tổng quan'!$E$38),"■","")</f>
         <v/>
       </c>
-      <c r="R29" s="24" t="str">
+      <c r="R29" s="23" t="str">
         <f>IF(AND(R$3&lt;='Timeline tổng quan'!$F$38,R$3+6&gt;='Timeline tổng quan'!$E$38),"■","")</f>
         <v/>
       </c>
-      <c r="S29" s="24" t="str">
+      <c r="S29" s="23" t="str">
         <f>IF(AND(S$3&lt;='Timeline tổng quan'!$F$38,S$3+6&gt;='Timeline tổng quan'!$E$38),"■","")</f>
         <v>■</v>
       </c>
-      <c r="T29" s="30" t="str">
+      <c r="T29" s="29" t="str">
         <f>IF(AND(T$3&lt;='Timeline tổng quan'!$F$38,T$3+6&gt;='Timeline tổng quan'!$E$38),"■","")</f>
         <v/>
       </c>
     </row>
     <row r="30" spans="1:20" ht="27" customHeight="1">
-      <c r="A30" s="31">
+      <c r="A30" s="30">
         <f>'Timeline tổng quan'!A39</f>
         <v>27</v>
       </c>
-      <c r="B30" s="32" t="str">
+      <c r="B30" s="31" t="str">
         <f>'Timeline tổng quan'!B39</f>
         <v>VI. ĐÓNG GÓI, TRÌNH BÀY &amp; DỰ PHÒNG</v>
       </c>
-      <c r="C30" s="32" t="str">
+      <c r="C30" s="31" t="str">
         <f>'Timeline tổng quan'!C39</f>
         <v>Nộp / bảo vệ / trình bày theo deadline</v>
       </c>
-      <c r="D30" s="32" t="str">
+      <c r="D30" s="31" t="str">
         <f>'Timeline tổng quan'!H39</f>
         <v>Chưa bắt đầu</v>
       </c>
-      <c r="E30" s="33" t="str">
+      <c r="E30" s="32" t="str">
         <f>IF(AND(E$3&lt;='Timeline tổng quan'!$F$39,E$3+6&gt;='Timeline tổng quan'!$E$39),"■","")</f>
         <v/>
       </c>
-      <c r="F30" s="33" t="str">
+      <c r="F30" s="32" t="str">
         <f>IF(AND(F$3&lt;='Timeline tổng quan'!$F$39,F$3+6&gt;='Timeline tổng quan'!$E$39),"■","")</f>
         <v/>
       </c>
-      <c r="G30" s="33" t="str">
+      <c r="G30" s="32" t="str">
         <f>IF(AND(G$3&lt;='Timeline tổng quan'!$F$39,G$3+6&gt;='Timeline tổng quan'!$E$39),"■","")</f>
         <v/>
       </c>
-      <c r="H30" s="33" t="str">
+      <c r="H30" s="32" t="str">
         <f>IF(AND(H$3&lt;='Timeline tổng quan'!$F$39,H$3+6&gt;='Timeline tổng quan'!$E$39),"■","")</f>
         <v/>
       </c>
-      <c r="I30" s="33" t="str">
+      <c r="I30" s="32" t="str">
         <f>IF(AND(I$3&lt;='Timeline tổng quan'!$F$39,I$3+6&gt;='Timeline tổng quan'!$E$39),"■","")</f>
         <v/>
       </c>
-      <c r="J30" s="33" t="str">
+      <c r="J30" s="32" t="str">
         <f>IF(AND(J$3&lt;='Timeline tổng quan'!$F$39,J$3+6&gt;='Timeline tổng quan'!$E$39),"■","")</f>
         <v/>
       </c>
-      <c r="K30" s="33" t="str">
+      <c r="K30" s="32" t="str">
         <f>IF(AND(K$3&lt;='Timeline tổng quan'!$F$39,K$3+6&gt;='Timeline tổng quan'!$E$39),"■","")</f>
         <v/>
       </c>
-      <c r="L30" s="33" t="str">
+      <c r="L30" s="32" t="str">
         <f>IF(AND(L$3&lt;='Timeline tổng quan'!$F$39,L$3+6&gt;='Timeline tổng quan'!$E$39),"■","")</f>
         <v/>
       </c>
-      <c r="M30" s="33" t="str">
+      <c r="M30" s="32" t="str">
         <f>IF(AND(M$3&lt;='Timeline tổng quan'!$F$39,M$3+6&gt;='Timeline tổng quan'!$E$39),"■","")</f>
         <v/>
       </c>
-      <c r="N30" s="33" t="str">
+      <c r="N30" s="32" t="str">
         <f>IF(AND(N$3&lt;='Timeline tổng quan'!$F$39,N$3+6&gt;='Timeline tổng quan'!$E$39),"■","")</f>
         <v/>
       </c>
-      <c r="O30" s="33" t="str">
+      <c r="O30" s="32" t="str">
         <f>IF(AND(O$3&lt;='Timeline tổng quan'!$F$39,O$3+6&gt;='Timeline tổng quan'!$E$39),"■","")</f>
         <v/>
       </c>
-      <c r="P30" s="33" t="str">
+      <c r="P30" s="32" t="str">
         <f>IF(AND(P$3&lt;='Timeline tổng quan'!$F$39,P$3+6&gt;='Timeline tổng quan'!$E$39),"■","")</f>
         <v/>
       </c>
-      <c r="Q30" s="33" t="str">
+      <c r="Q30" s="32" t="str">
         <f>IF(AND(Q$3&lt;='Timeline tổng quan'!$F$39,Q$3+6&gt;='Timeline tổng quan'!$E$39),"■","")</f>
         <v/>
       </c>
-      <c r="R30" s="33" t="str">
+      <c r="R30" s="32" t="str">
         <f>IF(AND(R$3&lt;='Timeline tổng quan'!$F$39,R$3+6&gt;='Timeline tổng quan'!$E$39),"■","")</f>
         <v/>
       </c>
-      <c r="S30" s="33" t="str">
+      <c r="S30" s="32" t="str">
         <f>IF(AND(S$3&lt;='Timeline tổng quan'!$F$39,S$3+6&gt;='Timeline tổng quan'!$E$39),"■","")</f>
         <v/>
       </c>
-      <c r="T30" s="34" t="str">
+      <c r="T30" s="33" t="str">
         <f>IF(AND(T$3&lt;='Timeline tổng quan'!$F$39,T$3+6&gt;='Timeline tổng quan'!$E$39),"■","")</f>
         <v>■</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="13.9" customHeight="1">
-      <c r="A33" s="75" t="s">
-        <v>191</v>
-      </c>
-      <c r="B33" s="48"/>
-      <c r="C33" s="48"/>
-      <c r="D33" s="48"/>
+      <c r="A33" s="69" t="s">
+        <v>192</v>
+      </c>
+      <c r="B33" s="70"/>
+      <c r="C33" s="70"/>
+      <c r="D33" s="70"/>
     </row>
     <row r="34" spans="1:4" ht="27" customHeight="1">
       <c r="A34" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C34" s="1"/>
       <c r="D34" s="1"/>
     </row>
     <row r="35" spans="1:4" ht="54" customHeight="1">
       <c r="A35" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D35" s="1"/>
     </row>
     <row r="36" spans="1:4" ht="27" customHeight="1">
       <c r="A36" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D36" s="1"/>
     </row>

</xml_diff>